<commit_message>
Deploying to gh-pages from  @ b219d0d034a2cca4f4f7bd94a0ccee18b942d1df 🚀
</commit_message>
<xml_diff>
--- a/Dic_Ausprägungen.xlsx
+++ b/Dic_Ausprägungen.xlsx
@@ -435,7 +435,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D397"/>
+  <dimension ref="A1:D409"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col customWidth="true" min="1" max="1" width="29.8828125"/>
@@ -5177,403 +5177,403 @@
     <row outlineLevel="0" r="216">
       <c r="A216" s="4" t="inlineStr">
         <is>
-          <t>A_RISKEXT_0</t>
+          <t>A_RECEIVER_COMM</t>
         </is>
       </c>
       <c r="B216" s="4" t="inlineStr">
         <is>
-          <t>K_RISKEXT</t>
+          <t>K_RECEIVER</t>
         </is>
       </c>
       <c r="C216" s="4" t="inlineStr">
         <is>
-          <t>Gefährdet</t>
+          <t>Handelsgesellschaften</t>
         </is>
       </c>
       <c r="D216" s="4" t="inlineStr">
         <is>
-          <t>At risk</t>
+          <t>Commercial company</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="217">
       <c r="A217" s="4" t="inlineStr">
         <is>
-          <t>A_RISKEXT_1</t>
+          <t>A_RECEIVER_GENEBANK</t>
         </is>
       </c>
       <c r="B217" s="4" t="inlineStr">
         <is>
-          <t>K_RISKEXT</t>
+          <t>K_RECEIVER</t>
         </is>
       </c>
       <c r="C217" s="4" t="inlineStr">
         <is>
-          <t>Nicht gefährdet</t>
+          <t>Gendatenbanken</t>
         </is>
       </c>
       <c r="D217" s="4" t="inlineStr">
         <is>
-          <t>Not at risk</t>
+          <t>Gene bank</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="218">
       <c r="A218" s="4" t="inlineStr">
         <is>
-          <t>A_RISKEXT_3</t>
+          <t>A_RECEIVER_INCREASE</t>
         </is>
       </c>
       <c r="B218" s="4" t="inlineStr">
         <is>
-          <t>K_RISKEXT</t>
+          <t>K_RECEIVER</t>
         </is>
       </c>
       <c r="C218" s="4" t="inlineStr">
         <is>
-          <t>Beobachtungspopulation</t>
+          <t>Projekt INCREASE</t>
         </is>
       </c>
       <c r="D218" s="4" t="inlineStr">
         <is>
-          <t>Monitoring Population</t>
+          <t>INCREASE project</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="219">
       <c r="A219" s="4" t="inlineStr">
         <is>
-          <t>A_RISKEXT_4</t>
+          <t>A_RECEIVER_INDIVID</t>
         </is>
       </c>
       <c r="B219" s="4" t="inlineStr">
         <is>
-          <t>K_RISKEXT</t>
+          <t>K_RECEIVER</t>
         </is>
       </c>
       <c r="C219" s="4" t="inlineStr">
         <is>
-          <t>Erhaltungspopulation</t>
+          <t>Einzelpersonen</t>
         </is>
       </c>
       <c r="D219" s="4" t="inlineStr">
         <is>
-          <t>Conservation Population</t>
+          <t>Individual</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="220">
       <c r="A220" s="4" t="inlineStr">
         <is>
-          <t>A_RISKEXT_6</t>
+          <t>A_RECEIVER_NONGOV</t>
         </is>
       </c>
       <c r="B220" s="4" t="inlineStr">
         <is>
-          <t>K_RISKEXT</t>
+          <t>K_RECEIVER</t>
         </is>
       </c>
       <c r="C220" s="4" t="inlineStr">
         <is>
-          <t>Phänotypische Erhaltungspopulation</t>
+          <t>Nichtregierungsorganisationen</t>
         </is>
       </c>
       <c r="D220" s="4" t="inlineStr">
         <is>
-          <t>Phenotypic Conservation Populations</t>
+          <t>Non-governmental organization</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="221">
       <c r="A221" s="4" t="inlineStr">
         <is>
-          <t>A_SANI</t>
+          <t>A_RECEIVER_OTHER</t>
         </is>
       </c>
       <c r="B221" s="4" t="inlineStr">
         <is>
-          <t>K_SERIES</t>
+          <t>K_RECEIVER</t>
         </is>
       </c>
       <c r="C221" s="4" t="inlineStr">
         <is>
-          <t>Wasser und Sanitär</t>
+          <t>Andere</t>
         </is>
       </c>
       <c r="D221" s="4" t="inlineStr">
         <is>
-          <t>Water and sanitation</t>
+          <t>Other</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="222">
       <c r="A222" s="4" t="inlineStr">
         <is>
-          <t>A_SCHUTZBEREICH_01</t>
+          <t>A_RECEIVER_REGIONORG</t>
         </is>
       </c>
       <c r="B222" s="4" t="inlineStr">
         <is>
-          <t>K_SCHUTZBEREICH</t>
+          <t>K_RECEIVER</t>
         </is>
       </c>
       <c r="C222" s="4" t="inlineStr">
         <is>
-          <t>Luft und Klima (CEP 01)</t>
+          <t>Regionale Organisationen</t>
         </is>
       </c>
       <c r="D222" s="4" t="inlineStr">
         <is>
-          <t>Air and climate (CEP 01)</t>
+          <t>Regional organization</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="223">
       <c r="A223" s="4" t="inlineStr">
         <is>
-          <t>A_SCHUTZBEREICH_02</t>
+          <t>A_RECEIVER_RESEARCH</t>
         </is>
       </c>
       <c r="B223" s="4" t="inlineStr">
         <is>
-          <t>K_SCHUTZBEREICH</t>
+          <t>K_RECEIVER</t>
         </is>
       </c>
       <c r="C223" s="4" t="inlineStr">
         <is>
-          <t>Energie aus erneuerbaren Quellen (CEP 0201)</t>
+          <t>Nationales Agrarforschungszentrum</t>
         </is>
       </c>
       <c r="D223" s="4" t="inlineStr">
         <is>
-          <t>Energy from renewable sources (CEP 0201)</t>
+          <t>National agricultural research centre</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="224">
       <c r="A224" s="4" t="inlineStr">
         <is>
-          <t>A_SCHUTZBEREICH_03</t>
+          <t>A_RECEIVER_UNI</t>
         </is>
       </c>
       <c r="B224" s="4" t="inlineStr">
         <is>
-          <t>K_SCHUTZBEREICH</t>
+          <t>K_RECEIVER</t>
         </is>
       </c>
       <c r="C224" s="4" t="inlineStr">
         <is>
-          <t>Energieeinsparungen und -management (CEP 0202)</t>
+          <t>Universitäten</t>
         </is>
       </c>
       <c r="D224" s="4" t="inlineStr">
         <is>
-          <t>Energy savings and management (CEP 0202)</t>
+          <t>University</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="225">
       <c r="A225" s="4" t="inlineStr">
         <is>
-          <t>A_SCHUTZBEREICH_04</t>
+          <t>A_RECEIVER_UNKNWN</t>
         </is>
       </c>
       <c r="B225" s="4" t="inlineStr">
         <is>
-          <t>K_SCHUTZBEREICH</t>
+          <t>K_RECEIVER</t>
         </is>
       </c>
       <c r="C225" s="4" t="inlineStr">
         <is>
-          <t>Abwasserwirtschaft (CEP 0301)</t>
+          <t>Unbekannt</t>
         </is>
       </c>
       <c r="D225" s="4" t="inlineStr">
         <is>
-          <t>Wastewater management (CEP 0301)</t>
+          <t>Unknown</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="226">
       <c r="A226" s="4" t="inlineStr">
         <is>
-          <t>A_SCHUTZBEREICH_05</t>
+          <t>A_RISKEXT_0</t>
         </is>
       </c>
       <c r="B226" s="4" t="inlineStr">
         <is>
-          <t>K_SCHUTZBEREICH</t>
+          <t>K_RISKEXT</t>
         </is>
       </c>
       <c r="C226" s="4" t="inlineStr">
         <is>
-          <t>Wassereinsparungen und Management der natürlichen Wasserressourcen (CEP 0302)</t>
+          <t>Gefährdet</t>
         </is>
       </c>
       <c r="D226" s="4" t="inlineStr">
         <is>
-          <t>Water savings and management of natural water resources (CEP 0302)</t>
+          <t>At risk</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="227">
       <c r="A227" s="4" t="inlineStr">
         <is>
-          <t>A_SCHUTZBEREICH_06</t>
+          <t>A_RISKEXT_1</t>
         </is>
       </c>
       <c r="B227" s="4" t="inlineStr">
         <is>
-          <t>K_SCHUTZBEREICH</t>
+          <t>K_RISKEXT</t>
         </is>
       </c>
       <c r="C227" s="4" t="inlineStr">
         <is>
-          <t>Abfallwirtschaft (CEP 0401)</t>
+          <t>Nicht gefährdet</t>
         </is>
       </c>
       <c r="D227" s="4" t="inlineStr">
         <is>
-          <t>Waste management (CEP 0401)</t>
+          <t>Not at risk</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="228">
       <c r="A228" s="4" t="inlineStr">
         <is>
-          <t>A_SCHUTZBEREICH_07</t>
+          <t>A_RISKEXT_3</t>
         </is>
       </c>
       <c r="B228" s="4" t="inlineStr">
         <is>
-          <t>K_SCHUTZBEREICH</t>
+          <t>K_RISKEXT</t>
         </is>
       </c>
       <c r="C228" s="4" t="inlineStr">
         <is>
-          <t>Wertstoffrückgewinnung und -einsparungen (CEP 0402)</t>
+          <t>Beobachtungspopulation</t>
         </is>
       </c>
       <c r="D228" s="4" t="inlineStr">
         <is>
-          <t>Materials recovery and savings (CEP 0402)</t>
+          <t>Monitoring Population</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="229">
       <c r="A229" s="4" t="inlineStr">
         <is>
-          <t>A_SCHUTZBEREICH_08</t>
+          <t>A_RISKEXT_4</t>
         </is>
       </c>
       <c r="B229" s="4" t="inlineStr">
         <is>
-          <t>K_SCHUTZBEREICH</t>
+          <t>K_RISKEXT</t>
         </is>
       </c>
       <c r="C229" s="4" t="inlineStr">
         <is>
-          <t>Schutz von Boden, Oberflächen- und Grundwasser (CEP 0501)</t>
+          <t>Erhaltungspopulation</t>
         </is>
       </c>
       <c r="D229" s="4" t="inlineStr">
         <is>
-          <t>Protection of soil, surface and groundwater (CEP 0501)</t>
+          <t>Conservation Population</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="230">
       <c r="A230" s="4" t="inlineStr">
         <is>
-          <t>A_SCHUTZBEREICH_09</t>
+          <t>A_RISKEXT_6</t>
         </is>
       </c>
       <c r="B230" s="4" t="inlineStr">
         <is>
-          <t>K_SCHUTZBEREICH</t>
+          <t>K_RISKEXT</t>
         </is>
       </c>
       <c r="C230" s="4" t="inlineStr">
         <is>
-          <t>Schutz von Biodiversität und Landschaft (CEP 0502)</t>
+          <t>Phänotypische Erhaltungspopulation</t>
         </is>
       </c>
       <c r="D230" s="4" t="inlineStr">
         <is>
-          <t>Protection of biodiversity and landscape (CEP 0502)</t>
+          <t>Phenotypic Conservation Populations</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="231">
       <c r="A231" s="4" t="inlineStr">
         <is>
-          <t>A_SCHUTZBEREICH_10</t>
+          <t>A_ROLE_REC</t>
         </is>
       </c>
       <c r="B231" s="4" t="inlineStr">
         <is>
-          <t>K_SCHUTZBEREICH</t>
+          <t>K_ROLE</t>
         </is>
       </c>
       <c r="C231" s="4" t="inlineStr">
         <is>
-          <t>Management von Waldressourcen (CEP 0503)</t>
+          <t>Empfänger</t>
         </is>
       </c>
       <c r="D231" s="4" t="inlineStr">
         <is>
-          <t>Management of forest resources (CEP 0503)</t>
+          <t>Receiver</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="232">
       <c r="A232" s="4" t="inlineStr">
         <is>
-          <t>A_SCHUTZBEREICH_11</t>
+          <t>A_ROLE_SND</t>
         </is>
       </c>
       <c r="B232" s="4" t="inlineStr">
         <is>
-          <t>K_SCHUTZBEREICH</t>
+          <t>K_ROLE</t>
         </is>
       </c>
       <c r="C232" s="4" t="inlineStr">
         <is>
-          <t>Lärm und Strahlung (CEP 06)</t>
+          <t>Bereitsteller</t>
         </is>
       </c>
       <c r="D232" s="4" t="inlineStr">
         <is>
-          <t>Noise and radiation (CEP 06)</t>
+          <t>Provider</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="233">
       <c r="A233" s="4" t="inlineStr">
         <is>
-          <t>A_SCHUTZBEREICH_12</t>
+          <t>A_SANI</t>
         </is>
       </c>
       <c r="B233" s="4" t="inlineStr">
         <is>
-          <t>K_SCHUTZBEREICH</t>
+          <t>K_SERIES</t>
         </is>
       </c>
       <c r="C233" s="4" t="inlineStr">
         <is>
-          <t>Forschung und Entwicklung auf dem Gebiet des Umweltschutzes (CEP 0701, 0703, 0705, 0707 und 0709)</t>
+          <t>Wasser und Sanitär</t>
         </is>
       </c>
       <c r="D233" s="4" t="inlineStr">
         <is>
-          <t>Research and development in the field of environmental protection (CEP 0701, 0703, 0705, 0707 und 0709)</t>
+          <t>Water and sanitation</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="234">
       <c r="A234" s="4" t="inlineStr">
         <is>
-          <t>A_SCHUTZBEREICH_13</t>
+          <t>A_SCHUTZBEREICH_01</t>
         </is>
       </c>
       <c r="B234" s="4" t="inlineStr">
@@ -5583,19 +5583,19 @@
       </c>
       <c r="C234" s="4" t="inlineStr">
         <is>
-          <t>Forschung und Entwicklung auf dem Gebiet des Ressourcenmanagements (CEP 0702, 0704, 0706 und 0708)</t>
+          <t>Luft und Klima (CEP 01)</t>
         </is>
       </c>
       <c r="D234" s="4" t="inlineStr">
         <is>
-          <t>Research and development in the field of resource management (CEP 0702, 0704, 0706 und 0708)</t>
+          <t>Air and climate (CEP 01)</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="235">
       <c r="A235" s="4" t="inlineStr">
         <is>
-          <t>A_SCHUTZBEREICH_14</t>
+          <t>A_SCHUTZBEREICH_02</t>
         </is>
       </c>
       <c r="B235" s="4" t="inlineStr">
@@ -5605,327 +5605,327 @@
       </c>
       <c r="C235" s="4" t="inlineStr">
         <is>
-          <t>Bereichsübergreifende Zwecke und andere Umweltzwecke (CEP 08)</t>
+          <t>Energie aus erneuerbaren Quellen (CEP 0201)</t>
         </is>
       </c>
       <c r="D235" s="4" t="inlineStr">
         <is>
-          <t>Cross-cutting and other environmental purposes (CEP 08)</t>
+          <t>Energy from renewable sources (CEP 0201)</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="236">
       <c r="A236" s="4" t="inlineStr">
         <is>
-          <t>A_SCORE_CURRENT</t>
+          <t>A_SCHUTZBEREICH_03</t>
         </is>
       </c>
       <c r="B236" s="4" t="inlineStr">
         <is>
-          <t>K_SCORE</t>
+          <t>K_SCHUTZBEREICH</t>
         </is>
       </c>
       <c r="C236" s="4" t="inlineStr">
         <is>
-          <t>Aktueller Stand</t>
+          <t>Energieeinsparungen und -management (CEP 0202)</t>
         </is>
       </c>
       <c r="D236" s="4" t="inlineStr">
         <is>
-          <t>Current status</t>
+          <t>Energy savings and management (CEP 0202)</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="237">
       <c r="A237" s="4" t="inlineStr">
         <is>
-          <t>A_SCORE_TREND</t>
+          <t>A_SCHUTZBEREICH_04</t>
         </is>
       </c>
       <c r="B237" s="4" t="inlineStr">
         <is>
-          <t>K_SCORE</t>
+          <t>K_SCHUTZBEREICH</t>
         </is>
       </c>
       <c r="C237" s="4" t="inlineStr">
         <is>
-          <t>Trend</t>
+          <t>Abwasserwirtschaft (CEP 0301)</t>
         </is>
       </c>
       <c r="D237" s="4" t="inlineStr">
         <is>
-          <t>Trend</t>
+          <t>Wastewater management (CEP 0301)</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="238">
       <c r="A238" s="4" t="inlineStr">
         <is>
-          <t>A_SDG_1</t>
+          <t>A_SCHUTZBEREICH_05</t>
         </is>
       </c>
       <c r="B238" s="4" t="inlineStr">
         <is>
-          <t>K_SDG</t>
+          <t>K_SCHUTZBEREICH</t>
         </is>
       </c>
       <c r="C238" s="4" t="inlineStr">
         <is>
-          <t>1 - Keine Armut</t>
+          <t>Wassereinsparungen und Management der natürlichen Wasserressourcen (CEP 0302)</t>
         </is>
       </c>
       <c r="D238" s="4" t="inlineStr">
         <is>
-          <t>1 - No poverty</t>
+          <t>Water savings and management of natural water resources (CEP 0302)</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="239">
       <c r="A239" s="4" t="inlineStr">
         <is>
-          <t>A_SDG_10</t>
+          <t>A_SCHUTZBEREICH_06</t>
         </is>
       </c>
       <c r="B239" s="4" t="inlineStr">
         <is>
-          <t>K_SDG</t>
+          <t>K_SCHUTZBEREICH</t>
         </is>
       </c>
       <c r="C239" s="4" t="inlineStr">
         <is>
-          <t>10 - Weniger Ungleichheiten</t>
+          <t>Abfallwirtschaft (CEP 0401)</t>
         </is>
       </c>
       <c r="D239" s="4" t="inlineStr">
         <is>
-          <t>10 - Reduced inequalities</t>
+          <t>Waste management (CEP 0401)</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="240">
       <c r="A240" s="4" t="inlineStr">
         <is>
-          <t>A_SDG_11</t>
+          <t>A_SCHUTZBEREICH_07</t>
         </is>
       </c>
       <c r="B240" s="4" t="inlineStr">
         <is>
-          <t>K_SDG</t>
+          <t>K_SCHUTZBEREICH</t>
         </is>
       </c>
       <c r="C240" s="4" t="inlineStr">
         <is>
-          <t>11 - Nachhaltige Städte und Gemeinden</t>
+          <t>Wertstoffrückgewinnung und -einsparungen (CEP 0402)</t>
         </is>
       </c>
       <c r="D240" s="4" t="inlineStr">
         <is>
-          <t>11 - Sustainable cities and communities</t>
+          <t>Materials recovery and savings (CEP 0402)</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="241">
       <c r="A241" s="4" t="inlineStr">
         <is>
-          <t>A_SDG_12</t>
+          <t>A_SCHUTZBEREICH_08</t>
         </is>
       </c>
       <c r="B241" s="4" t="inlineStr">
         <is>
-          <t>K_SDG</t>
+          <t>K_SCHUTZBEREICH</t>
         </is>
       </c>
       <c r="C241" s="4" t="inlineStr">
         <is>
-          <t>12 - Nachhaltige/r Konsum und Produktion</t>
+          <t>Schutz von Boden, Oberflächen- und Grundwasser (CEP 0501)</t>
         </is>
       </c>
       <c r="D241" s="4" t="inlineStr">
         <is>
-          <t>12 - Responsible consumption and production</t>
+          <t>Protection of soil, surface and groundwater (CEP 0501)</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="242">
       <c r="A242" s="4" t="inlineStr">
         <is>
-          <t>A_SDG_15</t>
+          <t>A_SCHUTZBEREICH_09</t>
         </is>
       </c>
       <c r="B242" s="4" t="inlineStr">
         <is>
-          <t>K_SDG</t>
+          <t>K_SCHUTZBEREICH</t>
         </is>
       </c>
       <c r="C242" s="4" t="inlineStr">
         <is>
-          <t>15 - Leben an Land</t>
+          <t>Schutz von Biodiversität und Landschaft (CEP 0502)</t>
         </is>
       </c>
       <c r="D242" s="4" t="inlineStr">
         <is>
-          <t>15 - Life on land</t>
+          <t>Protection of biodiversity and landscape (CEP 0502)</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="243">
       <c r="A243" s="4" t="inlineStr">
         <is>
-          <t>A_SDG_16</t>
+          <t>A_SCHUTZBEREICH_10</t>
         </is>
       </c>
       <c r="B243" s="4" t="inlineStr">
         <is>
-          <t>K_SDG</t>
+          <t>K_SCHUTZBEREICH</t>
         </is>
       </c>
       <c r="C243" s="4" t="inlineStr">
         <is>
-          <t>16 - Frieden, Gerechtigkeit und starke Institutionen</t>
+          <t>Management von Waldressourcen (CEP 0503)</t>
         </is>
       </c>
       <c r="D243" s="4" t="inlineStr">
         <is>
-          <t>16 - Peace and justice</t>
+          <t>Management of forest resources (CEP 0503)</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="244">
       <c r="A244" s="4" t="inlineStr">
         <is>
-          <t>A_SDG_17</t>
+          <t>A_SCHUTZBEREICH_11</t>
         </is>
       </c>
       <c r="B244" s="4" t="inlineStr">
         <is>
-          <t>K_SDG</t>
+          <t>K_SCHUTZBEREICH</t>
         </is>
       </c>
       <c r="C244" s="4" t="inlineStr">
         <is>
-          <t>17 - Partnerschaften zur Erreichung der Ziele</t>
+          <t>Lärm und Strahlung (CEP 06)</t>
         </is>
       </c>
       <c r="D244" s="4" t="inlineStr">
         <is>
-          <t>17 - Partnerships for the goals</t>
+          <t>Noise and radiation (CEP 06)</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="245">
       <c r="A245" s="4" t="inlineStr">
         <is>
-          <t>A_SDG_2</t>
+          <t>A_SCHUTZBEREICH_12</t>
         </is>
       </c>
       <c r="B245" s="4" t="inlineStr">
         <is>
-          <t>K_SDG</t>
+          <t>K_SCHUTZBEREICH</t>
         </is>
       </c>
       <c r="C245" s="4" t="inlineStr">
         <is>
-          <t>2 - Kein Hunger</t>
+          <t>Forschung und Entwicklung auf dem Gebiet des Umweltschutzes (CEP 0701, 0703, 0705, 0707 und 0709)</t>
         </is>
       </c>
       <c r="D245" s="4" t="inlineStr">
         <is>
-          <t>2 - Zero hunger</t>
+          <t>Research and development in the field of environmental protection (CEP 0701, 0703, 0705, 0707 und 0709)</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="246">
       <c r="A246" s="4" t="inlineStr">
         <is>
-          <t>A_SDG_3</t>
+          <t>A_SCHUTZBEREICH_13</t>
         </is>
       </c>
       <c r="B246" s="4" t="inlineStr">
         <is>
-          <t>K_SDG</t>
+          <t>K_SCHUTZBEREICH</t>
         </is>
       </c>
       <c r="C246" s="4" t="inlineStr">
         <is>
-          <t>3 - Gesundheit und Wohlergehen</t>
+          <t>Forschung und Entwicklung auf dem Gebiet des Ressourcenmanagements (CEP 0702, 0704, 0706 und 0708)</t>
         </is>
       </c>
       <c r="D246" s="4" t="inlineStr">
         <is>
-          <t>3 - Good health and well-being</t>
+          <t>Research and development in the field of resource management (CEP 0702, 0704, 0706 und 0708)</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="247">
       <c r="A247" s="4" t="inlineStr">
         <is>
-          <t>A_SDG_4</t>
+          <t>A_SCHUTZBEREICH_14</t>
         </is>
       </c>
       <c r="B247" s="4" t="inlineStr">
         <is>
-          <t>K_SDG</t>
+          <t>K_SCHUTZBEREICH</t>
         </is>
       </c>
       <c r="C247" s="4" t="inlineStr">
         <is>
-          <t>4 - Hochwertige Bildung</t>
+          <t>Bereichsübergreifende Zwecke und andere Umweltzwecke (CEP 08)</t>
         </is>
       </c>
       <c r="D247" s="4" t="inlineStr">
         <is>
-          <t>4 - Quality education</t>
+          <t>Cross-cutting and other environmental purposes (CEP 08)</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="248">
       <c r="A248" s="4" t="inlineStr">
         <is>
-          <t>A_SDG_5</t>
+          <t>A_SCORE_CURRENT</t>
         </is>
       </c>
       <c r="B248" s="4" t="inlineStr">
         <is>
-          <t>K_SDG</t>
+          <t>K_SCORE</t>
         </is>
       </c>
       <c r="C248" s="4" t="inlineStr">
         <is>
-          <t>5 - Geschlechtergleichheit</t>
+          <t>Aktueller Stand</t>
         </is>
       </c>
       <c r="D248" s="4" t="inlineStr">
         <is>
-          <t>5 - Gender equality</t>
+          <t>Current status</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="249">
       <c r="A249" s="4" t="inlineStr">
         <is>
-          <t>A_SDG_8</t>
+          <t>A_SCORE_TREND</t>
         </is>
       </c>
       <c r="B249" s="4" t="inlineStr">
         <is>
-          <t>K_SDG</t>
+          <t>K_SCORE</t>
         </is>
       </c>
       <c r="C249" s="4" t="inlineStr">
         <is>
-          <t>8 - Menschenwürdige Arbeit und Wirtschaftswachstum</t>
+          <t>Trend</t>
         </is>
       </c>
       <c r="D249" s="4" t="inlineStr">
         <is>
-          <t>8 - Decent work and economic Growth</t>
+          <t>Trend</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="250">
       <c r="A250" s="4" t="inlineStr">
         <is>
-          <t>A_SDG_9</t>
+          <t>A_SDG_1</t>
         </is>
       </c>
       <c r="B250" s="4" t="inlineStr">
@@ -5935,376 +5935,376 @@
       </c>
       <c r="C250" s="4" t="inlineStr">
         <is>
-          <t>9 - Industrie, Innovation und Infrastruktur</t>
+          <t>1 - Keine Armut</t>
         </is>
       </c>
       <c r="D250" s="4" t="inlineStr">
         <is>
-          <t>9 - Industry, innovation and infrastructure</t>
+          <t>1 - No poverty</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="251">
       <c r="A251" s="4" t="inlineStr">
         <is>
-          <t>A_SEA_B</t>
+          <t>A_SDG_10</t>
         </is>
       </c>
       <c r="B251" s="4" t="inlineStr">
         <is>
-          <t>K_SEA</t>
+          <t>K_SDG</t>
         </is>
       </c>
       <c r="C251" s="4" t="inlineStr">
         <is>
-          <t>Ostsee</t>
+          <t>10 - Weniger Ungleichheiten</t>
         </is>
       </c>
       <c r="D251" s="4" t="inlineStr">
         <is>
-          <t>Baltic sea</t>
+          <t>10 - Reduced inequalities</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="252">
       <c r="A252" s="4" t="inlineStr">
         <is>
-          <t>A_SEA_N</t>
+          <t>A_SDG_11</t>
         </is>
       </c>
       <c r="B252" s="4" t="inlineStr">
         <is>
-          <t>K_SEA</t>
+          <t>K_SDG</t>
         </is>
       </c>
       <c r="C252" s="4" t="inlineStr">
         <is>
-          <t>Nordsee</t>
+          <t>11 - Nachhaltige Städte und Gemeinden</t>
         </is>
       </c>
       <c r="D252" s="4" t="inlineStr">
         <is>
-          <t>Greater North Sea</t>
+          <t>11 - Sustainable cities and communities</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="253">
       <c r="A253" s="4" t="inlineStr">
         <is>
-          <t>A_SECTION_1</t>
+          <t>A_SDG_12</t>
         </is>
       </c>
       <c r="B253" s="4" t="inlineStr">
         <is>
-          <t>K_SECTION</t>
+          <t>K_SDG</t>
         </is>
       </c>
       <c r="C253" s="4" t="inlineStr">
         <is>
-          <t>Politische Führung und zentrale Verwaltung, Auswärtige Angelegenheiten</t>
+          <t>12 - Nachhaltige/r Konsum und Produktion</t>
         </is>
       </c>
       <c r="D253" s="4" t="inlineStr">
         <is>
-          <t>Political leadership and central administration, foreign affairs</t>
+          <t>12 - Responsible consumption and production</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="254">
       <c r="A254" s="4" t="inlineStr">
         <is>
-          <t>A_SECTION_2</t>
+          <t>A_SDG_15</t>
         </is>
       </c>
       <c r="B254" s="4" t="inlineStr">
         <is>
-          <t>K_SECTION</t>
+          <t>K_SDG</t>
         </is>
       </c>
       <c r="C254" s="4" t="inlineStr">
         <is>
-          <t>Polizei</t>
+          <t>15 - Leben an Land</t>
         </is>
       </c>
       <c r="D254" s="4" t="inlineStr">
         <is>
-          <t>Police</t>
+          <t>15 - Life on land</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="255">
       <c r="A255" s="4" t="inlineStr">
         <is>
-          <t>A_SECTION_3</t>
+          <t>A_SDG_16</t>
         </is>
       </c>
       <c r="B255" s="4" t="inlineStr">
         <is>
-          <t>K_SECTION</t>
+          <t>K_SDG</t>
         </is>
       </c>
       <c r="C255" s="4" t="inlineStr">
         <is>
-          <t>Bildungswesen, Wissenschaft, Forschung, kulturelle Angelegenheiten</t>
+          <t>16 - Frieden, Gerechtigkeit und starke Institutionen</t>
         </is>
       </c>
       <c r="D255" s="4" t="inlineStr">
         <is>
-          <t>Education, science, research, cultural affairs</t>
+          <t>16 - Peace and justice</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="256">
       <c r="A256" s="4" t="inlineStr">
         <is>
-          <t>A_SECTION_4</t>
+          <t>A_SDG_17</t>
         </is>
       </c>
       <c r="B256" s="4" t="inlineStr">
         <is>
-          <t>K_SECTION</t>
+          <t>K_SDG</t>
         </is>
       </c>
       <c r="C256" s="4" t="inlineStr">
         <is>
-          <t>Gesundheit, Umwelt, Sport und Erholung</t>
+          <t>17 - Partnerschaften zur Erreichung der Ziele</t>
         </is>
       </c>
       <c r="D256" s="4" t="inlineStr">
         <is>
-          <t>Health, environment, sports and recreation</t>
+          <t>17 - Partnerships for the goals</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="257">
       <c r="A257" s="4" t="inlineStr">
         <is>
-          <t>A_SECTIONS_0</t>
+          <t>A_SDG_2</t>
         </is>
       </c>
       <c r="B257" s="4" t="inlineStr">
         <is>
-          <t>K_SECTIONS</t>
+          <t>K_SDG</t>
         </is>
       </c>
       <c r="C257" s="4" t="inlineStr">
         <is>
-          <t>Endbewertung</t>
+          <t>2 - Kein Hunger</t>
         </is>
       </c>
       <c r="D257" s="4" t="inlineStr">
         <is>
-          <t>Finale Score</t>
+          <t>2 - Zero hunger</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="258">
       <c r="A258" s="4" t="inlineStr">
         <is>
-          <t>A_SECTIONS_1</t>
+          <t>A_SDG_3</t>
         </is>
       </c>
       <c r="B258" s="4" t="inlineStr">
         <is>
-          <t>K_SECTIONS</t>
+          <t>K_SDG</t>
         </is>
       </c>
       <c r="C258" s="4" t="inlineStr">
         <is>
-          <t>Rahmenbedingungen</t>
+          <t>3 - Gesundheit und Wohlergehen</t>
         </is>
       </c>
       <c r="D258" s="4" t="inlineStr">
         <is>
-          <t>Enabling environment</t>
+          <t>3 - Good health and well-being</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="259">
       <c r="A259" s="4" t="inlineStr">
         <is>
-          <t>A_SECTIONS_2</t>
+          <t>A_SDG_4</t>
         </is>
       </c>
       <c r="B259" s="4" t="inlineStr">
         <is>
-          <t>K_SECTIONS</t>
+          <t>K_SDG</t>
         </is>
       </c>
       <c r="C259" s="4" t="inlineStr">
         <is>
-          <t>Institutionen und Beteiligung</t>
+          <t>4 - Hochwertige Bildung</t>
         </is>
       </c>
       <c r="D259" s="4" t="inlineStr">
         <is>
-          <t>Institutions and participation</t>
+          <t>4 - Quality education</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="260">
       <c r="A260" s="4" t="inlineStr">
         <is>
-          <t>A_SECTIONS_3</t>
+          <t>A_SDG_5</t>
         </is>
       </c>
       <c r="B260" s="4" t="inlineStr">
         <is>
-          <t>K_SECTIONS</t>
+          <t>K_SDG</t>
         </is>
       </c>
       <c r="C260" s="4" t="inlineStr">
         <is>
-          <t>Managementinstrumente</t>
+          <t>5 - Geschlechtergleichheit</t>
         </is>
       </c>
       <c r="D260" s="4" t="inlineStr">
         <is>
-          <t>Management Instruments</t>
+          <t>5 - Gender equality</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="261">
       <c r="A261" s="4" t="inlineStr">
         <is>
-          <t>A_SECTIONS_4</t>
+          <t>A_SDG_8</t>
         </is>
       </c>
       <c r="B261" s="4" t="inlineStr">
         <is>
-          <t>K_SECTIONS</t>
+          <t>K_SDG</t>
         </is>
       </c>
       <c r="C261" s="4" t="inlineStr">
         <is>
-          <t>Finanzierung</t>
+          <t>8 - Menschenwürdige Arbeit und Wirtschaftswachstum</t>
         </is>
       </c>
       <c r="D261" s="4" t="inlineStr">
         <is>
-          <t>Financing</t>
+          <t>8 - Decent work and economic Growth</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="262">
       <c r="A262" s="4" t="inlineStr">
         <is>
-          <t>A_SEKTOR_1</t>
+          <t>A_SDG_9</t>
         </is>
       </c>
       <c r="B262" s="4" t="inlineStr">
         <is>
-          <t>K_SEKTOR</t>
+          <t>K_SDG</t>
         </is>
       </c>
       <c r="C262" s="4" t="inlineStr">
         <is>
-          <t>Staat</t>
+          <t>9 - Industrie, Innovation und Infrastruktur</t>
         </is>
       </c>
       <c r="D262" s="4" t="inlineStr">
         <is>
-          <t>General government</t>
+          <t>9 - Industry, innovation and infrastructure</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="263">
       <c r="A263" s="4" t="inlineStr">
         <is>
-          <t>A_SEKTOR_10</t>
+          <t>A_SEA_B</t>
         </is>
       </c>
       <c r="B263" s="4" t="inlineStr">
         <is>
-          <t>K_SEKTOR</t>
+          <t>K_SEA</t>
         </is>
       </c>
       <c r="C263" s="4" t="inlineStr">
         <is>
-          <t>Verkehrs- und Nachrichtenwesen</t>
+          <t>Ostsee</t>
         </is>
       </c>
       <c r="D263" s="4" t="inlineStr">
         <is>
-          <t>Transport and communications</t>
+          <t>Baltic sea</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="264">
       <c r="A264" s="4" t="inlineStr">
         <is>
-          <t>A_SEKTOR_11</t>
+          <t>A_SEA_N</t>
         </is>
       </c>
       <c r="B264" s="4" t="inlineStr">
         <is>
-          <t>K_SEKTOR</t>
+          <t>K_SEA</t>
         </is>
       </c>
       <c r="C264" s="4" t="inlineStr">
         <is>
-          <t>Wohnungswesen, Städtebau, Raumordnung und kommunale Gemeinschaftsdienste</t>
+          <t>Nordsee</t>
         </is>
       </c>
       <c r="D264" s="4" t="inlineStr">
         <is>
-          <t>Housing, urban development, regional planning and municipal community services</t>
+          <t>Greater North Sea</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="265">
       <c r="A265" s="4" t="inlineStr">
         <is>
-          <t>A_SEKTOR_2</t>
+          <t>A_SECTION_1</t>
         </is>
       </c>
       <c r="B265" s="4" t="inlineStr">
         <is>
-          <t>K_SEKTOR</t>
+          <t>K_SECTION</t>
         </is>
       </c>
       <c r="C265" s="4" t="inlineStr">
         <is>
-          <t>Unternehmen</t>
+          <t>Politische Führung und zentrale Verwaltung, Auswärtige Angelegenheiten</t>
         </is>
       </c>
       <c r="D265" s="4" t="inlineStr">
         <is>
-          <t>Corporations</t>
+          <t>Political leadership and central administration, foreign affairs</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="266">
       <c r="A266" s="4" t="inlineStr">
         <is>
-          <t>A_SEKTOR_3</t>
+          <t>A_SECTION_2</t>
         </is>
       </c>
       <c r="B266" s="4" t="inlineStr">
         <is>
-          <t>K_SEKTOR</t>
+          <t>K_SECTION</t>
         </is>
       </c>
       <c r="C266" s="4" t="inlineStr">
         <is>
-          <t>Allgemeine Dienste</t>
+          <t>Polizei</t>
         </is>
       </c>
       <c r="D266" s="4" t="inlineStr">
         <is>
-          <t>General services</t>
+          <t>Police</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="267">
       <c r="A267" s="4" t="inlineStr">
         <is>
-          <t>A_SEKTOR_4</t>
+          <t>A_SECTION_3</t>
         </is>
       </c>
       <c r="B267" s="4" t="inlineStr">
         <is>
-          <t>K_SEKTOR</t>
+          <t>K_SECTION</t>
         </is>
       </c>
       <c r="C267" s="4" t="inlineStr">
@@ -6321,887 +6321,887 @@
     <row outlineLevel="0" r="268">
       <c r="A268" s="4" t="inlineStr">
         <is>
-          <t>A_SEKTOR_5</t>
+          <t>A_SECTION_4</t>
         </is>
       </c>
       <c r="B268" s="4" t="inlineStr">
         <is>
-          <t>K_SEKTOR</t>
+          <t>K_SECTION</t>
         </is>
       </c>
       <c r="C268" s="4" t="inlineStr">
         <is>
-          <t>Energie- und Wasserwirtschaft, Gewerbe, Dienstleistungen</t>
+          <t>Gesundheit, Umwelt, Sport und Erholung</t>
         </is>
       </c>
       <c r="D268" s="4" t="inlineStr">
         <is>
-          <t>Energy and water management, trade, services</t>
+          <t>Health, environment, sports and recreation</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="269">
       <c r="A269" s="4" t="inlineStr">
         <is>
-          <t>A_SEKTOR_6</t>
+          <t>A_SECTIONS_0</t>
         </is>
       </c>
       <c r="B269" s="4" t="inlineStr">
         <is>
-          <t>K_SEKTOR</t>
+          <t>K_SECTIONS</t>
         </is>
       </c>
       <c r="C269" s="4" t="inlineStr">
         <is>
-          <t>Ernährung, Landwirtschaft und Forsten</t>
+          <t>Endbewertung</t>
         </is>
       </c>
       <c r="D269" s="4" t="inlineStr">
         <is>
-          <t>Food, agriculture and forestry</t>
+          <t>Finale Score</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="270">
       <c r="A270" s="4" t="inlineStr">
         <is>
-          <t>A_SEKTOR_7</t>
+          <t>A_SECTIONS_1</t>
         </is>
       </c>
       <c r="B270" s="4" t="inlineStr">
         <is>
-          <t>K_SEKTOR</t>
+          <t>K_SECTIONS</t>
         </is>
       </c>
       <c r="C270" s="4" t="inlineStr">
         <is>
-          <t>Finanzwirtschaft</t>
+          <t>Rahmenbedingungen</t>
         </is>
       </c>
       <c r="D270" s="4" t="inlineStr">
         <is>
-          <t>Financial services</t>
+          <t>Enabling environment</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="271">
       <c r="A271" s="4" t="inlineStr">
         <is>
-          <t>A_SEKTOR_8</t>
+          <t>A_SECTIONS_2</t>
         </is>
       </c>
       <c r="B271" s="4" t="inlineStr">
         <is>
-          <t>K_SEKTOR</t>
+          <t>K_SECTIONS</t>
         </is>
       </c>
       <c r="C271" s="4" t="inlineStr">
         <is>
-          <t>Gesundheit, Umwelt, Sport und Erholung</t>
+          <t>Institutionen und Beteiligung</t>
         </is>
       </c>
       <c r="D271" s="4" t="inlineStr">
         <is>
-          <t>Health, environment, sport and recreation</t>
+          <t>Institutions and participation</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="272">
       <c r="A272" s="4" t="inlineStr">
         <is>
-          <t>A_SEKTOR_9</t>
+          <t>A_SECTIONS_3</t>
         </is>
       </c>
       <c r="B272" s="4" t="inlineStr">
         <is>
-          <t>K_SEKTOR</t>
+          <t>K_SECTIONS</t>
         </is>
       </c>
       <c r="C272" s="4" t="inlineStr">
         <is>
-          <t>Soziale Sicherung, Familie und Jugend, Arbeitsmarktpolitik</t>
+          <t>Managementinstrumente</t>
         </is>
       </c>
       <c r="D272" s="4" t="inlineStr">
         <is>
-          <t>Social security, family and youth, labour market policy</t>
+          <t>Management Instruments</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="273">
       <c r="A273" s="4" t="inlineStr">
         <is>
-          <t>A_SERIES_DRCTTRANSFUND</t>
+          <t>A_SECTIONS_4</t>
         </is>
       </c>
       <c r="B273" s="4" t="inlineStr">
         <is>
-          <t>K_SERIES</t>
+          <t>K_SECTIONS</t>
         </is>
       </c>
       <c r="C273" s="4" t="inlineStr">
         <is>
-          <t>Direkte finanzielle Beihilfen</t>
+          <t>Finanzierung</t>
         </is>
       </c>
       <c r="D273" s="4" t="inlineStr">
         <is>
-          <t>Direct transfers of funds</t>
+          <t>Financing</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="274">
       <c r="A274" s="4" t="inlineStr">
         <is>
-          <t>A_SERIES_TAXBREAKS</t>
+          <t>A_SEKTOR_1</t>
         </is>
       </c>
       <c r="B274" s="4" t="inlineStr">
         <is>
-          <t>K_SERIES</t>
+          <t>K_SEKTOR</t>
         </is>
       </c>
       <c r="C274" s="4" t="inlineStr">
         <is>
-          <t>Steuervergünstigungen</t>
+          <t>Staat</t>
         </is>
       </c>
       <c r="D274" s="4" t="inlineStr">
         <is>
-          <t>Tax breaks</t>
+          <t>General government</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="275">
       <c r="A275" s="4" t="inlineStr">
         <is>
-          <t>A_SERIES_TOTAL</t>
+          <t>A_SEKTOR_10</t>
         </is>
       </c>
       <c r="B275" s="4" t="inlineStr">
         <is>
-          <t>K_SERIES</t>
+          <t>K_SEKTOR</t>
         </is>
       </c>
       <c r="C275" s="4" t="inlineStr">
         <is>
-          <t>Insgesamt</t>
+          <t>Verkehrs- und Nachrichtenwesen</t>
         </is>
       </c>
       <c r="D275" s="4" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Transport and communications</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="276">
       <c r="A276" s="4" t="inlineStr">
         <is>
-          <t>A_SEX_D</t>
+          <t>A_SEKTOR_11</t>
         </is>
       </c>
       <c r="B276" s="4" t="inlineStr">
         <is>
-          <t>K_SEX</t>
+          <t>K_SEKTOR</t>
         </is>
       </c>
       <c r="C276" s="4" t="inlineStr">
         <is>
-          <t>Divers</t>
+          <t>Wohnungswesen, Städtebau, Raumordnung und kommunale Gemeinschaftsdienste</t>
         </is>
       </c>
       <c r="D276" s="4" t="inlineStr">
         <is>
-          <t>Divers</t>
+          <t>Housing, urban development, regional planning and municipal community services</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="277">
       <c r="A277" s="4" t="inlineStr">
         <is>
-          <t>A_SEX_F</t>
+          <t>A_SEKTOR_2</t>
         </is>
       </c>
       <c r="B277" s="4" t="inlineStr">
         <is>
-          <t>K_SEX</t>
+          <t>K_SEKTOR</t>
         </is>
       </c>
       <c r="C277" s="4" t="inlineStr">
         <is>
-          <t>Weiblich</t>
+          <t>Unternehmen</t>
         </is>
       </c>
       <c r="D277" s="4" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Corporations</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="278">
       <c r="A278" s="4" t="inlineStr">
         <is>
-          <t>A_SEX_M</t>
+          <t>A_SEKTOR_3</t>
         </is>
       </c>
       <c r="B278" s="4" t="inlineStr">
         <is>
-          <t>K_SEX</t>
+          <t>K_SEKTOR</t>
         </is>
       </c>
       <c r="C278" s="4" t="inlineStr">
         <is>
-          <t>Männlich</t>
+          <t>Allgemeine Dienste</t>
         </is>
       </c>
       <c r="D278" s="4" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>General services</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="279">
       <c r="A279" s="4" t="inlineStr">
         <is>
-          <t>A_SEX_U</t>
+          <t>A_SEKTOR_4</t>
         </is>
       </c>
       <c r="B279" s="4" t="inlineStr">
         <is>
-          <t>K_SEX</t>
+          <t>K_SEKTOR</t>
         </is>
       </c>
       <c r="C279" s="4" t="inlineStr">
         <is>
-          <t>Unbekannt</t>
+          <t>Bildungswesen, Wissenschaft, Forschung, kulturelle Angelegenheiten</t>
         </is>
       </c>
       <c r="D279" s="4" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Education, science, research, cultural affairs</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="280">
       <c r="A280" s="4" t="inlineStr">
         <is>
-          <t>A_SKILL_1</t>
+          <t>A_SEKTOR_5</t>
         </is>
       </c>
       <c r="B280" s="4" t="inlineStr">
         <is>
-          <t>K_SKILL</t>
+          <t>K_SEKTOR</t>
         </is>
       </c>
       <c r="C280" s="4" t="inlineStr">
         <is>
-          <t>a) Lesen</t>
+          <t>Energie- und Wasserwirtschaft, Gewerbe, Dienstleistungen</t>
         </is>
       </c>
       <c r="D280" s="4" t="inlineStr">
         <is>
-          <t>a) Literacy skills</t>
+          <t>Energy and water management, trade, services</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="281">
       <c r="A281" s="4" t="inlineStr">
         <is>
-          <t>A_SKILL_2</t>
+          <t>A_SEKTOR_6</t>
         </is>
       </c>
       <c r="B281" s="4" t="inlineStr">
         <is>
-          <t>K_SKILL</t>
+          <t>K_SEKTOR</t>
         </is>
       </c>
       <c r="C281" s="4" t="inlineStr">
         <is>
-          <t>b) Rechnen</t>
+          <t>Ernährung, Landwirtschaft und Forsten</t>
         </is>
       </c>
       <c r="D281" s="4" t="inlineStr">
         <is>
-          <t>b) Numeracy skills</t>
+          <t>Food, agriculture and forestry</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="282">
       <c r="A282" s="4" t="inlineStr">
         <is>
-          <t>A_SOURCE_BMLEH</t>
+          <t>A_SEKTOR_7</t>
         </is>
       </c>
       <c r="B282" s="4" t="inlineStr">
         <is>
-          <t>K_SOURCE</t>
+          <t>K_SEKTOR</t>
         </is>
       </c>
       <c r="C282" s="4" t="inlineStr">
         <is>
-          <t>BMLEH</t>
+          <t>Finanzwirtschaft</t>
         </is>
       </c>
       <c r="D282" s="4" t="inlineStr">
         <is>
-          <t>Federal Ministry of Agriculture, Food and Regional Identity</t>
+          <t>Financial services</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="283">
       <c r="A283" s="4" t="inlineStr">
         <is>
-          <t>A_SOURCE_STBA</t>
+          <t>A_SEKTOR_8</t>
         </is>
       </c>
       <c r="B283" s="4" t="inlineStr">
         <is>
-          <t>K_SOURCE</t>
+          <t>K_SEKTOR</t>
         </is>
       </c>
       <c r="C283" s="4" t="inlineStr">
         <is>
-          <t>Statistisches Bundesamt</t>
+          <t>Gesundheit, Umwelt, Sport und Erholung</t>
         </is>
       </c>
       <c r="D283" s="4" t="inlineStr">
         <is>
-          <t>Federal Statistical Office</t>
+          <t>Health, environment, sport and recreation</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="284">
       <c r="A284" s="4" t="inlineStr">
         <is>
-          <t>A_SPEED_0</t>
+          <t>A_SEKTOR_9</t>
         </is>
       </c>
       <c r="B284" s="4" t="inlineStr">
         <is>
-          <t>K_SPEED</t>
+          <t>K_SEKTOR</t>
         </is>
       </c>
       <c r="C284" s="4" t="inlineStr">
         <is>
-          <t>a) Über 144 kbit/s bis unter 2 Mbit/s</t>
+          <t>Soziale Sicherung, Familie und Jugend, Arbeitsmarktpolitik</t>
         </is>
       </c>
       <c r="D284" s="4" t="inlineStr">
         <is>
-          <t>a) Over 144 kbps to under 2 mbps</t>
+          <t>Social security, family and youth, labour market policy</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="285">
       <c r="A285" s="4" t="inlineStr">
         <is>
-          <t>A_SPEED_1</t>
+          <t>A_SERIES_DRCTTRANSFUND</t>
         </is>
       </c>
       <c r="B285" s="4" t="inlineStr">
         <is>
-          <t>K_SPEED</t>
+          <t>K_SERIES</t>
         </is>
       </c>
       <c r="C285" s="4" t="inlineStr">
         <is>
-          <t>b) 2 Mbit/s bis unter 10 Mbit/s</t>
+          <t>Direkte finanzielle Beihilfen</t>
         </is>
       </c>
       <c r="D285" s="4" t="inlineStr">
         <is>
-          <t>b) 2 mbps to under 10 mbps</t>
+          <t>Direct transfers of funds</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="286">
       <c r="A286" s="4" t="inlineStr">
         <is>
-          <t>A_SPEED_2</t>
+          <t>A_SERIES_TAXBREAKS</t>
         </is>
       </c>
       <c r="B286" s="4" t="inlineStr">
         <is>
-          <t>K_SPEED</t>
+          <t>K_SERIES</t>
         </is>
       </c>
       <c r="C286" s="4" t="inlineStr">
         <is>
-          <t>c) 10 Mbit/s bis unter 30 Mbit/s</t>
+          <t>Steuervergünstigungen</t>
         </is>
       </c>
       <c r="D286" s="4" t="inlineStr">
         <is>
-          <t>c) 10 mbps to under 30 mbps</t>
+          <t>Tax breaks</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="287">
       <c r="A287" s="4" t="inlineStr">
         <is>
-          <t>A_SPEED_3</t>
+          <t>A_SERIES_TOTAL</t>
         </is>
       </c>
       <c r="B287" s="4" t="inlineStr">
         <is>
-          <t>K_SPEED</t>
+          <t>K_SERIES</t>
         </is>
       </c>
       <c r="C287" s="4" t="inlineStr">
         <is>
-          <t>d) 30 Mbit/s bis unter 100 Mbit/s</t>
+          <t>Insgesamt</t>
         </is>
       </c>
       <c r="D287" s="4" t="inlineStr">
         <is>
-          <t>d) 30 mbps to under 100 mbps</t>
+          <t>Total</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="288">
       <c r="A288" s="4" t="inlineStr">
         <is>
-          <t>A_SPEED_4</t>
+          <t>A_SEX_D</t>
         </is>
       </c>
       <c r="B288" s="4" t="inlineStr">
         <is>
-          <t>K_SPEED</t>
+          <t>K_SEX</t>
         </is>
       </c>
       <c r="C288" s="4" t="inlineStr">
         <is>
-          <t>e) 100 Mbit/s und mehr</t>
+          <t>Divers</t>
         </is>
       </c>
       <c r="D288" s="4" t="inlineStr">
         <is>
-          <t>e) 100 mbps and over</t>
+          <t>Divers</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="289">
       <c r="A289" s="4" t="inlineStr">
         <is>
-          <t>A_STDACCNTSYS_SEEA</t>
+          <t>A_SEX_F</t>
         </is>
       </c>
       <c r="B289" s="4" t="inlineStr">
         <is>
-          <t>K_STDACCNTSYS</t>
+          <t>K_SEX</t>
         </is>
       </c>
       <c r="C289" s="4" t="inlineStr">
         <is>
-          <t>SEEA Tabellen</t>
+          <t>Weiblich</t>
         </is>
       </c>
       <c r="D289" s="4" t="inlineStr">
         <is>
-          <t>SEEA tables</t>
+          <t>Female</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="290">
       <c r="A290" s="4" t="inlineStr">
         <is>
-          <t>A_STDACCNTSYS_TSA</t>
+          <t>A_SEX_M</t>
         </is>
       </c>
       <c r="B290" s="4" t="inlineStr">
         <is>
-          <t>K_STDACCNTSYS</t>
+          <t>K_SEX</t>
         </is>
       </c>
       <c r="C290" s="4" t="inlineStr">
         <is>
-          <t>TSA Tabellen</t>
+          <t>Männlich</t>
         </is>
       </c>
       <c r="D290" s="4" t="inlineStr">
         <is>
-          <t>TSA tables</t>
+          <t>Male</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="291">
       <c r="A291" s="4" t="inlineStr">
         <is>
-          <t>A_STIPENDIEN</t>
+          <t>A_SEX_U</t>
         </is>
       </c>
       <c r="B291" s="4" t="inlineStr">
         <is>
-          <t>K_SERIES</t>
+          <t>K_SEX</t>
         </is>
       </c>
       <c r="C291" s="4" t="inlineStr">
         <is>
-          <t>Stipendien</t>
+          <t>Unbekannt</t>
         </is>
       </c>
       <c r="D291" s="4" t="inlineStr">
         <is>
-          <t>Scholarships</t>
+          <t>Unknown</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="292">
       <c r="A292" s="4" t="inlineStr">
         <is>
-          <t>A_SUBJCT_0</t>
+          <t>A_SKILL_1</t>
         </is>
       </c>
       <c r="B292" s="4" t="inlineStr">
         <is>
-          <t>K_SUBJCT</t>
+          <t>K_SKILL</t>
         </is>
       </c>
       <c r="C292" s="4" t="inlineStr">
         <is>
-          <t>Lesen</t>
+          <t>a) Lesen</t>
         </is>
       </c>
       <c r="D292" s="4" t="inlineStr">
         <is>
-          <t>Reading</t>
+          <t>a) Literacy skills</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="293">
       <c r="A293" s="4" t="inlineStr">
         <is>
-          <t>A_SUBJCT_1</t>
+          <t>A_SKILL_2</t>
         </is>
       </c>
       <c r="B293" s="4" t="inlineStr">
         <is>
-          <t>K_SUBJCT</t>
+          <t>K_SKILL</t>
         </is>
       </c>
       <c r="C293" s="4" t="inlineStr">
         <is>
-          <t>Mathematik</t>
+          <t>b) Rechnen</t>
         </is>
       </c>
       <c r="D293" s="4" t="inlineStr">
         <is>
-          <t>Mathematics</t>
+          <t>b) Numeracy skills</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="294">
       <c r="A294" s="4" t="inlineStr">
         <is>
-          <t>A_SUBSTANCE_1</t>
+          <t>A_SOURCE_BMLEH</t>
         </is>
       </c>
       <c r="B294" s="4" t="inlineStr">
         <is>
-          <t>K_SUBSTANCE</t>
+          <t>K_SOURCE</t>
         </is>
       </c>
       <c r="C294" s="4" t="inlineStr">
         <is>
-          <t>Drogen</t>
+          <t>BMLEH</t>
         </is>
       </c>
       <c r="D294" s="4" t="inlineStr">
         <is>
-          <t>Drugs</t>
+          <t>Federal Ministry of Agriculture, Food and Regional Identity</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="295">
       <c r="A295" s="4" t="inlineStr">
         <is>
-          <t>A_SUBSTANCE_2</t>
+          <t>A_SOURCE_STBA</t>
         </is>
       </c>
       <c r="B295" s="4" t="inlineStr">
         <is>
-          <t>K_SUBSTANCE</t>
+          <t>K_SOURCE</t>
         </is>
       </c>
       <c r="C295" s="4" t="inlineStr">
         <is>
-          <t>Alkohol und andere psychoaktive Substanzen</t>
+          <t>Statistisches Bundesamt</t>
         </is>
       </c>
       <c r="D295" s="4" t="inlineStr">
         <is>
-          <t>Alcohol and other psychoactive substances</t>
+          <t>Federal Statistical Office</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="296">
       <c r="A296" s="4" t="inlineStr">
         <is>
-          <t>A_TAX</t>
+          <t>A_SPEED_0</t>
         </is>
       </c>
       <c r="B296" s="4" t="inlineStr">
         <is>
-          <t>K_SERIES</t>
+          <t>K_SPEED</t>
         </is>
       </c>
       <c r="C296" s="4" t="inlineStr">
         <is>
-          <t>Steuern</t>
+          <t>a) Über 144 kbit/s bis unter 2 Mbit/s</t>
         </is>
       </c>
       <c r="D296" s="4" t="inlineStr">
         <is>
-          <t>National taxes</t>
+          <t>a) Over 144 kbps to under 2 mbps</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="297">
       <c r="A297" s="4" t="inlineStr">
         <is>
-          <t>A_TAX_SOCIAL</t>
+          <t>A_SPEED_1</t>
         </is>
       </c>
       <c r="B297" s="4" t="inlineStr">
         <is>
-          <t>K_SERIES</t>
+          <t>K_SPEED</t>
         </is>
       </c>
       <c r="C297" s="4" t="inlineStr">
         <is>
-          <t>Steuern und Sozialversicherungsausgaben</t>
+          <t>b) 2 Mbit/s bis unter 10 Mbit/s</t>
         </is>
       </c>
       <c r="D297" s="4" t="inlineStr">
         <is>
-          <t>National taxes and insurance contributions</t>
+          <t>b) 2 mbps to under 10 mbps</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="298">
       <c r="A298" s="4" t="inlineStr">
         <is>
-          <t>A_TECHNO_1</t>
+          <t>A_SPEED_2</t>
         </is>
       </c>
       <c r="B298" s="4" t="inlineStr">
         <is>
-          <t>K_TECHNO</t>
+          <t>K_SPEED</t>
         </is>
       </c>
       <c r="C298" s="4" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>c) 10 Mbit/s bis unter 30 Mbit/s</t>
         </is>
       </c>
       <c r="D298" s="4" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>c) 10 mbps to under 30 mbps</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="299">
       <c r="A299" s="4" t="inlineStr">
         <is>
-          <t>A_TECHNO_2</t>
+          <t>A_SPEED_3</t>
         </is>
       </c>
       <c r="B299" s="4" t="inlineStr">
         <is>
-          <t>K_TECHNO</t>
+          <t>K_SPEED</t>
         </is>
       </c>
       <c r="C299" s="4" t="inlineStr">
         <is>
-          <t>LTE</t>
+          <t>d) 30 Mbit/s bis unter 100 Mbit/s</t>
         </is>
       </c>
       <c r="D299" s="4" t="inlineStr">
         <is>
-          <t>LTE</t>
+          <t>d) 30 mbps to under 100 mbps</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="300">
       <c r="A300" s="4" t="inlineStr">
         <is>
-          <t>A_TECHNO_3</t>
+          <t>A_SPEED_4</t>
         </is>
       </c>
       <c r="B300" s="4" t="inlineStr">
         <is>
-          <t>K_TECHNO</t>
+          <t>K_SPEED</t>
         </is>
       </c>
       <c r="C300" s="4" t="inlineStr">
         <is>
-          <t>5G</t>
+          <t>e) 100 Mbit/s und mehr</t>
         </is>
       </c>
       <c r="D300" s="4" t="inlineStr">
         <is>
-          <t>5G</t>
+          <t>e) 100 mbps and over</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="301">
       <c r="A301" s="4" t="inlineStr">
         <is>
-          <t>A_TECHNOINT_1</t>
+          <t>A_STDACCNTSYS_SEEA</t>
         </is>
       </c>
       <c r="B301" s="4" t="inlineStr">
         <is>
-          <t>K_TECHNOINT</t>
+          <t>K_STDACCNTSYS</t>
         </is>
       </c>
       <c r="C301" s="4" t="inlineStr">
         <is>
-          <t>Medium-High-Tech</t>
+          <t>SEEA Tabellen</t>
         </is>
       </c>
       <c r="D301" s="4" t="inlineStr">
         <is>
-          <t>Medium-high-tech</t>
+          <t>SEEA tables</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="302">
       <c r="A302" s="4" t="inlineStr">
         <is>
-          <t>A_TECHNOINT_2</t>
+          <t>A_STDACCNTSYS_TSA</t>
         </is>
       </c>
       <c r="B302" s="4" t="inlineStr">
         <is>
-          <t>K_TECHNOINT</t>
+          <t>K_STDACCNTSYS</t>
         </is>
       </c>
       <c r="C302" s="4" t="inlineStr">
         <is>
-          <t>High-Tech</t>
+          <t>TSA Tabellen</t>
         </is>
       </c>
       <c r="D302" s="4" t="inlineStr">
         <is>
-          <t>High-tech</t>
+          <t>TSA tables</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="303">
       <c r="A303" s="4" t="inlineStr">
         <is>
-          <t>A_THEMATICAREA_1</t>
+          <t>A_STIPENDIEN</t>
         </is>
       </c>
       <c r="B303" s="4" t="inlineStr">
         <is>
-          <t>K_THEMATICAREA</t>
+          <t>K_SERIES</t>
         </is>
       </c>
       <c r="C303" s="4" t="inlineStr">
         <is>
-          <t>Bereich 1: Mutterschaftsvorsorge</t>
+          <t>Stipendien</t>
         </is>
       </c>
       <c r="D303" s="4" t="inlineStr">
         <is>
-          <t>Section 1: Maternity care</t>
+          <t>Scholarships</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="304">
       <c r="A304" s="4" t="inlineStr">
         <is>
-          <t>A_THEMATICAREA_2</t>
+          <t>A_SUBJCT_0</t>
         </is>
       </c>
       <c r="B304" s="4" t="inlineStr">
         <is>
-          <t>K_THEMATICAREA</t>
+          <t>K_SUBJCT</t>
         </is>
       </c>
       <c r="C304" s="4" t="inlineStr">
         <is>
-          <t>Bereich 2: Empfängnisverhütung und Familienplanung</t>
+          <t>Lesen</t>
         </is>
       </c>
       <c r="D304" s="4" t="inlineStr">
         <is>
-          <t>Section 2: Contraception and family planning</t>
+          <t>Reading</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="305">
       <c r="A305" s="4" t="inlineStr">
         <is>
-          <t>A_THEMATICAREA_3</t>
+          <t>A_SUBJCT_1</t>
         </is>
       </c>
       <c r="B305" s="4" t="inlineStr">
         <is>
-          <t>K_THEMATICAREA</t>
+          <t>K_SUBJCT</t>
         </is>
       </c>
       <c r="C305" s="4" t="inlineStr">
         <is>
-          <t>Bereich 3: Umfassende Sexualerziehung und Information</t>
+          <t>Mathematik</t>
         </is>
       </c>
       <c r="D305" s="4" t="inlineStr">
         <is>
-          <t>Section 3: Comprehensive sexuality education and information</t>
+          <t>Mathematics</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="306">
       <c r="A306" s="4" t="inlineStr">
         <is>
-          <t>A_THEMATICAREA_4</t>
+          <t>A_SUBSTANCE_1</t>
         </is>
       </c>
       <c r="B306" s="4" t="inlineStr">
         <is>
-          <t>K_THEMATICAREA</t>
+          <t>K_SUBSTANCE</t>
         </is>
       </c>
       <c r="C306" s="4" t="inlineStr">
         <is>
-          <t>Bereich 4: HIV und HPV</t>
+          <t>Drogen</t>
         </is>
       </c>
       <c r="D306" s="4" t="inlineStr">
         <is>
-          <t>Section 4: HIV and HPV</t>
+          <t>Drugs</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="307">
       <c r="A307" s="4" t="inlineStr">
         <is>
-          <t>A_TOURIS_EMPLOY</t>
+          <t>A_SUBSTANCE_2</t>
         </is>
       </c>
       <c r="B307" s="4" t="inlineStr">
         <is>
-          <t>K_SERIES</t>
+          <t>K_SUBSTANCE</t>
         </is>
       </c>
       <c r="C307" s="4" t="inlineStr">
         <is>
-          <t>&lt;u&gt;Zusätzliche Zeitreihe:&lt;/u&gt; Beschäftigte</t>
+          <t>Alkohol und andere psychoaktive Substanzen</t>
         </is>
       </c>
       <c r="D307" s="4" t="inlineStr">
         <is>
-          <t>&lt;u&gt;Additional time series:&lt;/u&gt; Employees</t>
+          <t>Alcohol and other psychoactive substances</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="308">
       <c r="A308" s="4" t="inlineStr">
         <is>
-          <t>A_TOURIS_JOB</t>
+          <t>A_TAX</t>
         </is>
       </c>
       <c r="B308" s="4" t="inlineStr">
@@ -7211,19 +7211,19 @@
       </c>
       <c r="C308" s="4" t="inlineStr">
         <is>
-          <t>&lt;u&gt;Zusätzliche Zeitreihe:&lt;/u&gt; Vollzeitäquivalente</t>
+          <t>Steuern</t>
         </is>
       </c>
       <c r="D308" s="4" t="inlineStr">
         <is>
-          <t>&lt;u&gt;Additional time series:&lt;/u&gt; Full-time equivalents</t>
+          <t>National taxes</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="309">
       <c r="A309" s="4" t="inlineStr">
         <is>
-          <t>A_TOURIS_PERSON</t>
+          <t>A_TAX_SOCIAL</t>
         </is>
       </c>
       <c r="B309" s="4" t="inlineStr">
@@ -7233,701 +7233,701 @@
       </c>
       <c r="C309" s="4" t="inlineStr">
         <is>
-          <t>&lt;u&gt;Zeitreihe des Indikators:&lt;/u&gt; Erwerbstätige</t>
+          <t>Steuern und Sozialversicherungsausgaben</t>
         </is>
       </c>
       <c r="D309" s="4" t="inlineStr">
         <is>
-          <t>&lt;u&gt;Time series of the indicator:&lt;/u&gt; Employed persons</t>
+          <t>National taxes and insurance contributions</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="310">
       <c r="A310" s="4" t="inlineStr">
         <is>
-          <t>A_TOURISINDUS_10</t>
+          <t>A_TECHNO_1</t>
         </is>
       </c>
       <c r="B310" s="4" t="inlineStr">
         <is>
-          <t>K_ECONSEC</t>
+          <t>K_TECHNO</t>
         </is>
       </c>
       <c r="C310" s="4" t="inlineStr">
         <is>
-          <t>Dienstleistungen des Sports und der Erholung</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="D310" s="4" t="inlineStr">
         <is>
-          <t>Sports and Recreational activities</t>
+          <t>3G</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="311">
       <c r="A311" s="4" t="inlineStr">
         <is>
-          <t>A_TOURISINDUS_1a</t>
+          <t>A_TECHNO_2</t>
         </is>
       </c>
       <c r="B311" s="4" t="inlineStr">
         <is>
-          <t>K_ECONSEC</t>
+          <t>K_TECHNO</t>
         </is>
       </c>
       <c r="C311" s="4" t="inlineStr">
         <is>
-          <t>Beherbergung: Hotels und ähnliche Beherbergungsstätten</t>
+          <t>LTE</t>
         </is>
       </c>
       <c r="D311" s="4" t="inlineStr">
         <is>
-          <t>Accommodation for visitors: hotels and similar establishments</t>
+          <t>LTE</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="312">
       <c r="A312" s="4" t="inlineStr">
         <is>
-          <t>A_TOURISINDUS_1b</t>
+          <t>A_TECHNO_3</t>
         </is>
       </c>
       <c r="B312" s="4" t="inlineStr">
         <is>
-          <t>K_ECONSEC</t>
+          <t>K_TECHNO</t>
         </is>
       </c>
       <c r="C312" s="4" t="inlineStr">
         <is>
-          <t>Beherbergung: Sonstige Beherbergungsstätten</t>
+          <t>5G</t>
         </is>
       </c>
       <c r="D312" s="4" t="inlineStr">
         <is>
-          <t>Accommodation for visitors: other</t>
+          <t>5G</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="313">
       <c r="A313" s="4" t="inlineStr">
         <is>
-          <t>A_TOURISINDUS_2</t>
+          <t>A_TECHNOINT_1</t>
         </is>
       </c>
       <c r="B313" s="4" t="inlineStr">
         <is>
-          <t>K_ECONSEC</t>
+          <t>K_TECHNOINT</t>
         </is>
       </c>
       <c r="C313" s="4" t="inlineStr">
         <is>
-          <t>Gaststätten- und Getränkeausschank</t>
+          <t>Medium-High-Tech</t>
         </is>
       </c>
       <c r="D313" s="4" t="inlineStr">
         <is>
-          <t>Food and beverage serving activities</t>
+          <t>Medium-high-tech</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="314">
       <c r="A314" s="4" t="inlineStr">
         <is>
-          <t>A_TOURISINDUS_3</t>
+          <t>A_TECHNOINT_2</t>
         </is>
       </c>
       <c r="B314" s="4" t="inlineStr">
         <is>
-          <t>K_ECONSEC</t>
+          <t>K_TECHNOINT</t>
         </is>
       </c>
       <c r="C314" s="4" t="inlineStr">
         <is>
-          <t>Personenbeförderung im Eisenbahnverkehr</t>
+          <t>High-Tech</t>
         </is>
       </c>
       <c r="D314" s="4" t="inlineStr">
         <is>
-          <t>Railway passenger transport</t>
+          <t>High-tech</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="315">
       <c r="A315" s="4" t="inlineStr">
         <is>
-          <t>A_TOURISINDUS_4</t>
+          <t>A_THEMATICAREA_1</t>
         </is>
       </c>
       <c r="B315" s="4" t="inlineStr">
         <is>
-          <t>K_ECONSEC</t>
+          <t>K_THEMATICAREA</t>
         </is>
       </c>
       <c r="C315" s="4" t="inlineStr">
         <is>
-          <t>Personenbeförderung im Straßenverkehr</t>
+          <t>Bereich 1: Mutterschaftsvorsorge</t>
         </is>
       </c>
       <c r="D315" s="4" t="inlineStr">
         <is>
-          <t>Road passenger transport</t>
+          <t>Section 1: Maternity care</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="316">
       <c r="A316" s="4" t="inlineStr">
         <is>
-          <t>A_TOURISINDUS_5</t>
+          <t>A_THEMATICAREA_2</t>
         </is>
       </c>
       <c r="B316" s="4" t="inlineStr">
         <is>
-          <t>K_ECONSEC</t>
+          <t>K_THEMATICAREA</t>
         </is>
       </c>
       <c r="C316" s="4" t="inlineStr">
         <is>
-          <t>Personenbeförderung in der Schifffahrt</t>
+          <t>Bereich 2: Empfängnisverhütung und Familienplanung</t>
         </is>
       </c>
       <c r="D316" s="4" t="inlineStr">
         <is>
-          <t>Water passenger transport</t>
+          <t>Section 2: Contraception and family planning</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="317">
       <c r="A317" s="4" t="inlineStr">
         <is>
-          <t>A_TOURISINDUS_6</t>
+          <t>A_THEMATICAREA_3</t>
         </is>
       </c>
       <c r="B317" s="4" t="inlineStr">
         <is>
-          <t>K_ECONSEC</t>
+          <t>K_THEMATICAREA</t>
         </is>
       </c>
       <c r="C317" s="4" t="inlineStr">
         <is>
-          <t>Personenbeförderung in der Luftfahrt</t>
+          <t>Bereich 3: Umfassende Sexualerziehung und Information</t>
         </is>
       </c>
       <c r="D317" s="4" t="inlineStr">
         <is>
-          <t>Air passenger transport</t>
+          <t>Section 3: Comprehensive sexuality education and information</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="318">
       <c r="A318" s="4" t="inlineStr">
         <is>
-          <t>A_TOURISINDUS_7</t>
+          <t>A_THEMATICAREA_4</t>
         </is>
       </c>
       <c r="B318" s="4" t="inlineStr">
         <is>
-          <t>K_ECONSEC</t>
+          <t>K_THEMATICAREA</t>
         </is>
       </c>
       <c r="C318" s="4" t="inlineStr">
         <is>
-          <t>Vermietung von Transportmitteln</t>
+          <t>Bereich 4: HIV und HPV</t>
         </is>
       </c>
       <c r="D318" s="4" t="inlineStr">
         <is>
-          <t>Transport equipment rental</t>
+          <t>Section 4: HIV and HPV</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="319">
       <c r="A319" s="4" t="inlineStr">
         <is>
-          <t>A_TOURISINDUS_8</t>
+          <t>A_TOURIS_EMPLOY</t>
         </is>
       </c>
       <c r="B319" s="4" t="inlineStr">
         <is>
-          <t>K_ECONSEC</t>
+          <t>K_SERIES</t>
         </is>
       </c>
       <c r="C319" s="4" t="inlineStr">
         <is>
-          <t>Reisebüros, Reiseveranstalter und sonstige Reservierungsdienstleistungen</t>
+          <t>&lt;u&gt;Zusätzliche Zeitreihe:&lt;/u&gt; Beschäftigte</t>
         </is>
       </c>
       <c r="D319" s="4" t="inlineStr">
         <is>
-          <t>Travel agencies and other reservation service activities</t>
+          <t>&lt;u&gt;Additional time series:&lt;/u&gt; Employees</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="320">
       <c r="A320" s="4" t="inlineStr">
         <is>
-          <t>A_TOURISINDUS_9</t>
+          <t>A_TOURIS_JOB</t>
         </is>
       </c>
       <c r="B320" s="4" t="inlineStr">
         <is>
-          <t>K_ECONSEC</t>
+          <t>K_SERIES</t>
         </is>
       </c>
       <c r="C320" s="4" t="inlineStr">
         <is>
-          <t>Kulturelle Dienstleistungen</t>
+          <t>&lt;u&gt;Zusätzliche Zeitreihe:&lt;/u&gt; Vollzeitäquivalente</t>
         </is>
       </c>
       <c r="D320" s="4" t="inlineStr">
         <is>
-          <t>Cultural activities</t>
+          <t>&lt;u&gt;Additional time series:&lt;/u&gt; Full-time equivalents</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="321">
       <c r="A321" s="4" t="inlineStr">
         <is>
-          <t>A_TRANSPTY_0</t>
+          <t>A_TOURIS_PERSON</t>
         </is>
       </c>
       <c r="B321" s="4" t="inlineStr">
         <is>
-          <t>K_TRANSPTY</t>
+          <t>K_SERIES</t>
         </is>
       </c>
       <c r="C321" s="4" t="inlineStr">
         <is>
-          <t>Binnenschifffahrt</t>
+          <t>&lt;u&gt;Zeitreihe des Indikators:&lt;/u&gt; Erwerbstätige</t>
         </is>
       </c>
       <c r="D321" s="4" t="inlineStr">
         <is>
-          <t>Inland waterway transport</t>
+          <t>&lt;u&gt;Time series of the indicator:&lt;/u&gt; Employed persons</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="322">
       <c r="A322" s="4" t="inlineStr">
         <is>
-          <t>A_TRANSPTY_1</t>
+          <t>A_TOURISINDUS_10</t>
         </is>
       </c>
       <c r="B322" s="4" t="inlineStr">
         <is>
-          <t>K_TRANSPTY</t>
+          <t>K_ECONSEC</t>
         </is>
       </c>
       <c r="C322" s="4" t="inlineStr">
         <is>
-          <t>Eisenbahnverkehr</t>
+          <t>Dienstleistungen des Sports und der Erholung</t>
         </is>
       </c>
       <c r="D322" s="4" t="inlineStr">
         <is>
-          <t>Rail transport</t>
+          <t>Sports and Recreational activities</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="323">
       <c r="A323" s="4" t="inlineStr">
         <is>
-          <t>A_TRANSPTY_2</t>
+          <t>A_TOURISINDUS_1a</t>
         </is>
       </c>
       <c r="B323" s="4" t="inlineStr">
         <is>
-          <t>K_TRANSPTY</t>
+          <t>K_ECONSEC</t>
         </is>
       </c>
       <c r="C323" s="4" t="inlineStr">
         <is>
-          <t>Luftverkehr</t>
+          <t>Beherbergung: Hotels und ähnliche Beherbergungsstätten</t>
         </is>
       </c>
       <c r="D323" s="4" t="inlineStr">
         <is>
-          <t>Air transport</t>
+          <t>Accommodation for visitors: hotels and similar establishments</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="324">
       <c r="A324" s="4" t="inlineStr">
         <is>
-          <t>A_TRANSPTY_3</t>
+          <t>A_TOURISINDUS_1b</t>
         </is>
       </c>
       <c r="B324" s="4" t="inlineStr">
         <is>
-          <t>K_TRANSPTY</t>
+          <t>K_ECONSEC</t>
         </is>
       </c>
       <c r="C324" s="4" t="inlineStr">
         <is>
-          <t>Motorisierter Individualverkehr</t>
+          <t>Beherbergung: Sonstige Beherbergungsstätten</t>
         </is>
       </c>
       <c r="D324" s="4" t="inlineStr">
         <is>
-          <t>Motorised private transport</t>
+          <t>Accommodation for visitors: other</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="325">
       <c r="A325" s="4" t="inlineStr">
         <is>
-          <t>A_TRANSPTY_4</t>
+          <t>A_TOURISINDUS_2</t>
         </is>
       </c>
       <c r="B325" s="4" t="inlineStr">
         <is>
-          <t>K_TRANSPTY</t>
+          <t>K_ECONSEC</t>
         </is>
       </c>
       <c r="C325" s="4" t="inlineStr">
         <is>
-          <t>Straßenverkehr</t>
+          <t>Gaststätten- und Getränkeausschank</t>
         </is>
       </c>
       <c r="D325" s="4" t="inlineStr">
         <is>
-          <t>Road transport</t>
+          <t>Food and beverage serving activities</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="326">
       <c r="A326" s="4" t="inlineStr">
         <is>
-          <t>A_TRANSPTY_5</t>
+          <t>A_TOURISINDUS_3</t>
         </is>
       </c>
       <c r="B326" s="4" t="inlineStr">
         <is>
-          <t>K_TRANSPTY</t>
+          <t>K_ECONSEC</t>
         </is>
       </c>
       <c r="C326" s="4" t="inlineStr">
         <is>
-          <t>Rohrfernleitungen: Rohöl</t>
+          <t>Personenbeförderung im Eisenbahnverkehr</t>
         </is>
       </c>
       <c r="D326" s="4" t="inlineStr">
         <is>
-          <t>Pipelines: crude oil</t>
+          <t>Railway passenger transport</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="327">
       <c r="A327" s="4" t="inlineStr">
         <is>
-          <t>A_TROP_BEH_BEDARF</t>
+          <t>A_TOURISINDUS_4</t>
         </is>
       </c>
       <c r="B327" s="4" t="inlineStr">
         <is>
-          <t>K_SERIES</t>
+          <t>K_ECONSEC</t>
         </is>
       </c>
       <c r="C327" s="4" t="inlineStr">
         <is>
-          <t>Personen mit Behandlungsbedarf</t>
+          <t>Personenbeförderung im Straßenverkehr</t>
         </is>
       </c>
       <c r="D327" s="4" t="inlineStr">
         <is>
-          <t>People requiring interventions</t>
+          <t>Road passenger transport</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="328">
       <c r="A328" s="4" t="inlineStr">
         <is>
-          <t>A_TROP_STAT_BEH</t>
+          <t>A_TOURISINDUS_5</t>
         </is>
       </c>
       <c r="B328" s="4" t="inlineStr">
         <is>
-          <t>K_SERIES</t>
+          <t>K_ECONSEC</t>
         </is>
       </c>
       <c r="C328" s="4" t="inlineStr">
         <is>
-          <t>Stationäre Behandlung</t>
+          <t>Personenbeförderung in der Schifffahrt</t>
         </is>
       </c>
       <c r="D328" s="4" t="inlineStr">
         <is>
-          <t>Inpatient treatment</t>
+          <t>Water passenger transport</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="329">
       <c r="A329" s="4" t="inlineStr">
         <is>
-          <t>A_TYPDISEASE_1</t>
+          <t>A_TOURISINDUS_6</t>
         </is>
       </c>
       <c r="B329" s="4" t="inlineStr">
         <is>
-          <t>K_TYPDISEASE</t>
+          <t>K_ECONSEC</t>
         </is>
       </c>
       <c r="C329" s="4" t="inlineStr">
         <is>
-          <t>a) Herz-Kreislauferkrankungen</t>
+          <t>Personenbeförderung in der Luftfahrt</t>
         </is>
       </c>
       <c r="D329" s="4" t="inlineStr">
         <is>
-          <t>a) Cardiovascular disease</t>
+          <t>Air passenger transport</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="330">
       <c r="A330" s="4" t="inlineStr">
         <is>
-          <t>A_TYPDISEASE_10</t>
+          <t>A_TOURISINDUS_7</t>
         </is>
       </c>
       <c r="B330" s="4" t="inlineStr">
         <is>
-          <t>K_TYPDISEASE</t>
+          <t>K_ECONSEC</t>
         </is>
       </c>
       <c r="C330" s="4" t="inlineStr">
         <is>
-          <t>Lepra</t>
+          <t>Vermietung von Transportmitteln</t>
         </is>
       </c>
       <c r="D330" s="4" t="inlineStr">
         <is>
-          <t>Leprosy</t>
+          <t>Transport equipment rental</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="331">
       <c r="A331" s="4" t="inlineStr">
         <is>
-          <t>A_TYPDISEASE_11</t>
+          <t>A_TOURISINDUS_8</t>
         </is>
       </c>
       <c r="B331" s="4" t="inlineStr">
         <is>
-          <t>K_TYPDISEASE</t>
+          <t>K_ECONSEC</t>
         </is>
       </c>
       <c r="C331" s="4" t="inlineStr">
         <is>
-          <t>Buruli-Ulkus</t>
+          <t>Reisebüros, Reiseveranstalter und sonstige Reservierungsdienstleistungen</t>
         </is>
       </c>
       <c r="D331" s="4" t="inlineStr">
         <is>
-          <t>Buruli ulcer</t>
+          <t>Travel agencies and other reservation service activities</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="332">
       <c r="A332" s="4" t="inlineStr">
         <is>
-          <t>A_TYPDISEASE_12</t>
+          <t>A_TOURISINDUS_9</t>
         </is>
       </c>
       <c r="B332" s="4" t="inlineStr">
         <is>
-          <t>K_TYPDISEASE</t>
+          <t>K_ECONSEC</t>
         </is>
       </c>
       <c r="C332" s="4" t="inlineStr">
         <is>
-          <t>Afrikanische Trypanosomiasis</t>
+          <t>Kulturelle Dienstleistungen</t>
         </is>
       </c>
       <c r="D332" s="4" t="inlineStr">
         <is>
-          <t>Human African Trypanosomiasis</t>
+          <t>Cultural activities</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="333">
       <c r="A333" s="4" t="inlineStr">
         <is>
-          <t>A_TYPDISEASE_13</t>
+          <t>A_TRANSPTY_0</t>
         </is>
       </c>
       <c r="B333" s="4" t="inlineStr">
         <is>
-          <t>K_TYPDISEASE</t>
+          <t>K_TRANSPTY</t>
         </is>
       </c>
       <c r="C333" s="4" t="inlineStr">
         <is>
-          <t>Leishmaniose</t>
+          <t>Binnenschifffahrt</t>
         </is>
       </c>
       <c r="D333" s="4" t="inlineStr">
         <is>
-          <t>Leishmaniases</t>
+          <t>Inland waterway transport</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="334">
       <c r="A334" s="4" t="inlineStr">
         <is>
-          <t>A_TYPDISEASE_14</t>
+          <t>A_TRANSPTY_1</t>
         </is>
       </c>
       <c r="B334" s="4" t="inlineStr">
         <is>
-          <t>K_TYPDISEASE</t>
+          <t>K_TRANSPTY</t>
         </is>
       </c>
       <c r="C334" s="4" t="inlineStr">
         <is>
-          <t>Tollwut</t>
+          <t>Eisenbahnverkehr</t>
         </is>
       </c>
       <c r="D334" s="4" t="inlineStr">
         <is>
-          <t>Rabies</t>
+          <t>Rail transport</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="335">
       <c r="A335" s="4" t="inlineStr">
         <is>
-          <t>A_TYPDISEASE_15</t>
+          <t>A_TRANSPTY_2</t>
         </is>
       </c>
       <c r="B335" s="4" t="inlineStr">
         <is>
-          <t>K_TYPDISEASE</t>
+          <t>K_TRANSPTY</t>
         </is>
       </c>
       <c r="C335" s="4" t="inlineStr">
         <is>
-          <t>Frambösie</t>
+          <t>Luftverkehr</t>
         </is>
       </c>
       <c r="D335" s="4" t="inlineStr">
         <is>
-          <t>Yaws</t>
+          <t>Air transport</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="336">
       <c r="A336" s="4" t="inlineStr">
         <is>
-          <t>A_TYPDISEASE_16</t>
+          <t>A_TRANSPTY_3</t>
         </is>
       </c>
       <c r="B336" s="4" t="inlineStr">
         <is>
-          <t>K_TYPDISEASE</t>
+          <t>K_TRANSPTY</t>
         </is>
       </c>
       <c r="C336" s="4" t="inlineStr">
         <is>
-          <t>Drakunkulose</t>
+          <t>Motorisierter Individualverkehr</t>
         </is>
       </c>
       <c r="D336" s="4" t="inlineStr">
         <is>
-          <t>Dracunculiasis</t>
+          <t>Motorised private transport</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="337">
       <c r="A337" s="4" t="inlineStr">
         <is>
-          <t>A_TYPDISEASE_17</t>
+          <t>A_TRANSPTY_4</t>
         </is>
       </c>
       <c r="B337" s="4" t="inlineStr">
         <is>
-          <t>K_TYPDISEASE</t>
+          <t>K_TRANSPTY</t>
         </is>
       </c>
       <c r="C337" s="4" t="inlineStr">
         <is>
-          <t>Chronisch obstruktive Lungenerkrankung (COPD)</t>
+          <t>Straßenverkehr</t>
         </is>
       </c>
       <c r="D337" s="4" t="inlineStr">
         <is>
-          <t>Chronic obstructive pulmonary disease (COPD)</t>
+          <t>Road transport</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="338">
       <c r="A338" s="4" t="inlineStr">
         <is>
-          <t>A_TYPDISEASE_18</t>
+          <t>A_TRANSPTY_5</t>
         </is>
       </c>
       <c r="B338" s="4" t="inlineStr">
         <is>
-          <t>K_TYPDISEASE</t>
+          <t>K_TRANSPTY</t>
         </is>
       </c>
       <c r="C338" s="4" t="inlineStr">
         <is>
-          <t>Lungenkrebs</t>
+          <t>Rohrfernleitungen: Rohöl</t>
         </is>
       </c>
       <c r="D338" s="4" t="inlineStr">
         <is>
-          <t>Lung cancer</t>
+          <t>Pipelines: crude oil</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="339">
       <c r="A339" s="4" t="inlineStr">
         <is>
-          <t>A_TYPDISEASE_19</t>
+          <t>A_TROP_BEH_BEDARF</t>
         </is>
       </c>
       <c r="B339" s="4" t="inlineStr">
         <is>
-          <t>K_TYPDISEASE</t>
+          <t>K_SERIES</t>
         </is>
       </c>
       <c r="C339" s="4" t="inlineStr">
         <is>
-          <t>Schlaganfall</t>
+          <t>Personen mit Behandlungsbedarf</t>
         </is>
       </c>
       <c r="D339" s="4" t="inlineStr">
         <is>
-          <t>Stroke</t>
+          <t>People requiring interventions</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="340">
       <c r="A340" s="4" t="inlineStr">
         <is>
-          <t>A_TYPDISEASE_2</t>
+          <t>A_TROP_STAT_BEH</t>
         </is>
       </c>
       <c r="B340" s="4" t="inlineStr">
         <is>
-          <t>K_TYPDISEASE</t>
+          <t>K_SERIES</t>
         </is>
       </c>
       <c r="C340" s="4" t="inlineStr">
         <is>
-          <t>b) Bösartige Neubildungen</t>
+          <t>Stationäre Behandlung</t>
         </is>
       </c>
       <c r="D340" s="4" t="inlineStr">
         <is>
-          <t>b) Cancer</t>
+          <t>Inpatient treatment</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="341">
       <c r="A341" s="4" t="inlineStr">
         <is>
-          <t>A_TYPDISEASE_20</t>
+          <t>A_TYPDISEASE_1</t>
         </is>
       </c>
       <c r="B341" s="4" t="inlineStr">
@@ -7937,19 +7937,19 @@
       </c>
       <c r="C341" s="4" t="inlineStr">
         <is>
-          <t>Ischämische Herzerkrankungen</t>
+          <t>a) Herz-Kreislauferkrankungen</t>
         </is>
       </c>
       <c r="D341" s="4" t="inlineStr">
         <is>
-          <t>Ischemic heart diseases</t>
+          <t>a) Cardiovascular disease</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="342">
       <c r="A342" s="4" t="inlineStr">
         <is>
-          <t>A_TYPDISEASE_21</t>
+          <t>A_TYPDISEASE_10</t>
         </is>
       </c>
       <c r="B342" s="4" t="inlineStr">
@@ -7959,19 +7959,19 @@
       </c>
       <c r="C342" s="4" t="inlineStr">
         <is>
-          <t>Diabetes mellitus Typ 2</t>
+          <t>Lepra</t>
         </is>
       </c>
       <c r="D342" s="4" t="inlineStr">
         <is>
-          <t>Diabetes mellitus type 2</t>
+          <t>Leprosy</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="343">
       <c r="A343" s="4" t="inlineStr">
         <is>
-          <t>A_TYPDISEASE_22</t>
+          <t>A_TYPDISEASE_11</t>
         </is>
       </c>
       <c r="B343" s="4" t="inlineStr">
@@ -7981,19 +7981,19 @@
       </c>
       <c r="C343" s="4" t="inlineStr">
         <is>
-          <t>a) Akute Atemwegsinfektionen</t>
+          <t>Buruli-Ulkus</t>
         </is>
       </c>
       <c r="D343" s="4" t="inlineStr">
         <is>
-          <t>a) Acute respiratory infections</t>
+          <t>Buruli ulcer</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="344">
       <c r="A344" s="4" t="inlineStr">
         <is>
-          <t>A_TYPDISEASE_3</t>
+          <t>A_TYPDISEASE_12</t>
         </is>
       </c>
       <c r="B344" s="4" t="inlineStr">
@@ -8003,19 +8003,19 @@
       </c>
       <c r="C344" s="4" t="inlineStr">
         <is>
-          <t>c) Diabetes mellitus</t>
+          <t>Afrikanische Trypanosomiasis</t>
         </is>
       </c>
       <c r="D344" s="4" t="inlineStr">
         <is>
-          <t>c) Diabetes mellitus</t>
+          <t>Human African Trypanosomiasis</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="345">
       <c r="A345" s="4" t="inlineStr">
         <is>
-          <t>A_TYPDISEASE_4</t>
+          <t>A_TYPDISEASE_13</t>
         </is>
       </c>
       <c r="B345" s="4" t="inlineStr">
@@ -8025,19 +8025,19 @@
       </c>
       <c r="C345" s="4" t="inlineStr">
         <is>
-          <t>d) Chronische Atemwegserkrankungen</t>
+          <t>Leishmaniose</t>
         </is>
       </c>
       <c r="D345" s="4" t="inlineStr">
         <is>
-          <t>d) Chronic respiratory disease</t>
+          <t>Leishmaniases</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="346">
       <c r="A346" s="4" t="inlineStr">
         <is>
-          <t>A_TYPDISEASE_5</t>
+          <t>A_TYPDISEASE_14</t>
         </is>
       </c>
       <c r="B346" s="4" t="inlineStr">
@@ -8047,19 +8047,19 @@
       </c>
       <c r="C346" s="4" t="inlineStr">
         <is>
-          <t>b) Durchfallerkrankungen</t>
+          <t>Tollwut</t>
         </is>
       </c>
       <c r="D346" s="4" t="inlineStr">
         <is>
-          <t>b) Diarrhoea</t>
+          <t>Rabies</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="347">
       <c r="A347" s="4" t="inlineStr">
         <is>
-          <t>A_TYPDISEASE_6</t>
+          <t>A_TYPDISEASE_15</t>
         </is>
       </c>
       <c r="B347" s="4" t="inlineStr">
@@ -8069,19 +8069,19 @@
       </c>
       <c r="C347" s="4" t="inlineStr">
         <is>
-          <t>c) Intestinale Nematodeninfektionen</t>
+          <t>Frambösie</t>
         </is>
       </c>
       <c r="D347" s="4" t="inlineStr">
         <is>
-          <t>c) Intestinal nematode infections</t>
+          <t>Yaws</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="348">
       <c r="A348" s="4" t="inlineStr">
         <is>
-          <t>A_TYPDISEASE_7</t>
+          <t>A_TYPDISEASE_16</t>
         </is>
       </c>
       <c r="B348" s="4" t="inlineStr">
@@ -8091,19 +8091,19 @@
       </c>
       <c r="C348" s="4" t="inlineStr">
         <is>
-          <t>d) Energie- und Eiweißmangelernährung</t>
+          <t>Drakunkulose</t>
         </is>
       </c>
       <c r="D348" s="4" t="inlineStr">
         <is>
-          <t>d) Protein-energy malnutrition</t>
+          <t>Dracunculiasis</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="349">
       <c r="A349" s="4" t="inlineStr">
         <is>
-          <t>A_TYPDISEASE_8</t>
+          <t>A_TYPDISEASE_17</t>
         </is>
       </c>
       <c r="B349" s="4" t="inlineStr">
@@ -8113,19 +8113,19 @@
       </c>
       <c r="C349" s="4" t="inlineStr">
         <is>
-          <t>Dengue</t>
+          <t>Chronisch obstruktive Lungenerkrankung (COPD)</t>
         </is>
       </c>
       <c r="D349" s="4" t="inlineStr">
         <is>
-          <t>Dengue</t>
+          <t>Chronic obstructive pulmonary disease (COPD)</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="350">
       <c r="A350" s="4" t="inlineStr">
         <is>
-          <t>A_TYPDISEASE_9</t>
+          <t>A_TYPDISEASE_18</t>
         </is>
       </c>
       <c r="B350" s="4" t="inlineStr">
@@ -8135,1044 +8135,1308 @@
       </c>
       <c r="C350" s="4" t="inlineStr">
         <is>
-          <t>Echinokokkose</t>
+          <t>Lungenkrebs</t>
         </is>
       </c>
       <c r="D350" s="4" t="inlineStr">
         <is>
-          <t>Echinococcosis</t>
+          <t>Lung cancer</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="351">
       <c r="A351" s="4" t="inlineStr">
         <is>
-          <t>A_TYPEABUSE_1</t>
+          <t>A_TYPDISEASE_19</t>
         </is>
       </c>
       <c r="B351" s="4" t="inlineStr">
         <is>
-          <t>K_TYPEABUSE</t>
+          <t>K_TYPDISEASE</t>
         </is>
       </c>
       <c r="C351" s="4" t="inlineStr">
         <is>
-          <t>Körperliche Misshandlung</t>
+          <t>Schlaganfall</t>
         </is>
       </c>
       <c r="D351" s="4" t="inlineStr">
         <is>
-          <t>Physical abuse</t>
+          <t>Stroke</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="352">
       <c r="A352" s="4" t="inlineStr">
         <is>
-          <t>A_TYPEABUSE_2</t>
+          <t>A_TYPDISEASE_2</t>
         </is>
       </c>
       <c r="B352" s="4" t="inlineStr">
         <is>
-          <t>K_TYPEABUSE</t>
+          <t>K_TYPDISEASE</t>
         </is>
       </c>
       <c r="C352" s="4" t="inlineStr">
         <is>
-          <t>Psychische Misshandlung</t>
+          <t>b) Bösartige Neubildungen</t>
         </is>
       </c>
       <c r="D352" s="4" t="inlineStr">
         <is>
-          <t>Psychological abuse</t>
+          <t>b) Cancer</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="353">
       <c r="A353" s="4" t="inlineStr">
         <is>
-          <t>A_TYPEACCOUNT_0</t>
+          <t>A_TYPDISEASE_20</t>
         </is>
       </c>
       <c r="B353" s="4" t="inlineStr">
         <is>
-          <t>K_TYPEACCOUNT</t>
+          <t>K_TYPDISEASE</t>
         </is>
       </c>
       <c r="C353" s="4" t="inlineStr">
         <is>
-          <t>Girokonten</t>
+          <t>Ischämische Herzerkrankungen</t>
         </is>
       </c>
       <c r="D353" s="4" t="inlineStr">
         <is>
-          <t>Current accounts</t>
+          <t>Ischemic heart diseases</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="354">
       <c r="A354" s="4" t="inlineStr">
         <is>
-          <t>A_TYPEACCOUNT_1</t>
+          <t>A_TYPDISEASE_21</t>
         </is>
       </c>
       <c r="B354" s="4" t="inlineStr">
         <is>
-          <t>K_TYPEACCOUNT</t>
+          <t>K_TYPDISEASE</t>
         </is>
       </c>
       <c r="C354" s="4" t="inlineStr">
         <is>
-          <t>Online-Konten</t>
+          <t>Diabetes mellitus Typ 2</t>
         </is>
       </c>
       <c r="D354" s="4" t="inlineStr">
         <is>
-          <t>Online accounts</t>
+          <t>Diabetes mellitus type 2</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="355">
       <c r="A355" s="4" t="inlineStr">
         <is>
-          <t>A_TYPEBIOMASS_1</t>
+          <t>A_TYPDISEASE_22</t>
         </is>
       </c>
       <c r="B355" s="4" t="inlineStr">
         <is>
-          <t>K_TYPEBIOMASS</t>
+          <t>K_TYPDISEASE</t>
         </is>
       </c>
       <c r="C355" s="4" t="inlineStr">
         <is>
-          <t>Stehendes Holz</t>
+          <t>a) Akute Atemwegsinfektionen</t>
         </is>
       </c>
       <c r="D355" s="4" t="inlineStr">
         <is>
-          <t>Standig wood</t>
+          <t>a) Acute respiratory infections</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="356">
       <c r="A356" s="4" t="inlineStr">
         <is>
-          <t>A_TYPEBIOMASS_2</t>
+          <t>A_TYPDISEASE_3</t>
         </is>
       </c>
       <c r="B356" s="4" t="inlineStr">
         <is>
-          <t>K_TYPEBIOMASS</t>
+          <t>K_TYPDISEASE</t>
         </is>
       </c>
       <c r="C356" s="4" t="inlineStr">
         <is>
-          <t>Sonstige Holzbiomasse</t>
+          <t>c) Diabetes mellitus</t>
         </is>
       </c>
       <c r="D356" s="4" t="inlineStr">
         <is>
-          <t>Other woody biomass</t>
+          <t>c) Diabetes mellitus</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="357">
       <c r="A357" s="4" t="inlineStr">
         <is>
-          <t>A_TYPEBIOMASS_3</t>
+          <t>A_TYPDISEASE_4</t>
         </is>
       </c>
       <c r="B357" s="4" t="inlineStr">
         <is>
-          <t>K_TYPEBIOMASS</t>
+          <t>K_TYPDISEASE</t>
         </is>
       </c>
       <c r="C357" s="4" t="inlineStr">
         <is>
-          <t>Sonstige Biomasse in Wäldern</t>
+          <t>d) Chronische Atemwegserkrankungen</t>
         </is>
       </c>
       <c r="D357" s="4" t="inlineStr">
         <is>
-          <t>Other biomass in forests</t>
+          <t>d) Chronic respiratory disease</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="358">
       <c r="A358" s="4" t="inlineStr">
         <is>
-          <t>A_TYPECLASS_FAO</t>
+          <t>A_TYPDISEASE_5</t>
         </is>
       </c>
       <c r="B358" s="4" t="inlineStr">
         <is>
-          <t>K_TYPECLASS</t>
+          <t>K_TYPDISEASE</t>
         </is>
       </c>
       <c r="C358" s="4" t="inlineStr">
         <is>
-          <t>FAO-Klassifikation</t>
+          <t>b) Durchfallerkrankungen</t>
         </is>
       </c>
       <c r="D358" s="4" t="inlineStr">
         <is>
-          <t>FAO classification</t>
+          <t>b) Diarrhoea</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="359">
       <c r="A359" s="4" t="inlineStr">
         <is>
-          <t>A_TYPECLASS_NAT</t>
+          <t>A_TYPDISEASE_6</t>
         </is>
       </c>
       <c r="B359" s="4" t="inlineStr">
         <is>
-          <t>K_TYPECLASS</t>
+          <t>K_TYPDISEASE</t>
         </is>
       </c>
       <c r="C359" s="4" t="inlineStr">
         <is>
-          <t>Nationale Klassifikation</t>
+          <t>c) Intestinale Nematodeninfektionen</t>
         </is>
       </c>
       <c r="D359" s="4" t="inlineStr">
         <is>
-          <t>National classification</t>
+          <t>c) Intestinal nematode infections</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="360">
       <c r="A360" s="4" t="inlineStr">
         <is>
-          <t>A_TYPEEXPLOITATION_1</t>
+          <t>A_TYPDISEASE_7</t>
         </is>
       </c>
       <c r="B360" s="4" t="inlineStr">
         <is>
-          <t>K_TYPEEXPLOITATION</t>
+          <t>K_TYPDISEASE</t>
         </is>
       </c>
       <c r="C360" s="4" t="inlineStr">
         <is>
-          <t>Ausbeutung der Arbeitskraft</t>
+          <t>d) Energie- und Eiweißmangelernährung</t>
         </is>
       </c>
       <c r="D360" s="4" t="inlineStr">
         <is>
-          <t>Labour exploitation</t>
+          <t>d) Protein-energy malnutrition</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="361">
       <c r="A361" s="4" t="inlineStr">
         <is>
-          <t>A_TYPEEXPLOITATION_2</t>
+          <t>A_TYPDISEASE_8</t>
         </is>
       </c>
       <c r="B361" s="4" t="inlineStr">
         <is>
-          <t>K_TYPEEXPLOITATION</t>
+          <t>K_TYPDISEASE</t>
         </is>
       </c>
       <c r="C361" s="4" t="inlineStr">
         <is>
-          <t>Sexuelle Ausbeutung</t>
+          <t>Dengue</t>
         </is>
       </c>
       <c r="D361" s="4" t="inlineStr">
         <is>
-          <t>Sexual exploitation</t>
+          <t>Dengue</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="362">
       <c r="A362" s="4" t="inlineStr">
         <is>
-          <t>A_TYPEFLOW_0</t>
+          <t>A_TYPDISEASE_9</t>
         </is>
       </c>
       <c r="B362" s="4" t="inlineStr">
         <is>
-          <t>K_TYPEFLOW</t>
+          <t>K_TYPDISEASE</t>
         </is>
       </c>
       <c r="C362" s="4" t="inlineStr">
         <is>
-          <t>Sonstige öffentliche Nettoausgaben (OOF)</t>
+          <t>Echinokokkose</t>
         </is>
       </c>
       <c r="D362" s="4" t="inlineStr">
         <is>
-          <t>OOF (net disbursements)</t>
+          <t>Echinococcosis</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="363">
       <c r="A363" s="4" t="inlineStr">
         <is>
-          <t>A_TYPEFLOW_1</t>
+          <t>A_TYPEABUSE_1</t>
         </is>
       </c>
       <c r="B363" s="4" t="inlineStr">
         <is>
-          <t>K_TYPEFLOW</t>
+          <t>K_TYPEABUSE</t>
         </is>
       </c>
       <c r="C363" s="4" t="inlineStr">
         <is>
-          <t>Öffentlich unterstützte Exportkredite (Nettoausgaben)</t>
+          <t>Körperliche Misshandlung</t>
         </is>
       </c>
       <c r="D363" s="4" t="inlineStr">
         <is>
-          <t>Officially supported export credits (net disbursements)</t>
+          <t>Physical abuse</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="364">
       <c r="A364" s="4" t="inlineStr">
         <is>
-          <t>A_TYPEFLOW_2</t>
+          <t>A_TYPEABUSE_2</t>
         </is>
       </c>
       <c r="B364" s="4" t="inlineStr">
         <is>
-          <t>K_TYPEFLOW</t>
+          <t>K_TYPEABUSE</t>
         </is>
       </c>
       <c r="C364" s="4" t="inlineStr">
         <is>
-          <t>Öffentliche Nettoentwicklungsausgaben (ODA)</t>
+          <t>Psychische Misshandlung</t>
         </is>
       </c>
       <c r="D364" s="4" t="inlineStr">
         <is>
-          <t>ODA (net disbursements)</t>
+          <t>Psychological abuse</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="365">
       <c r="A365" s="4" t="inlineStr">
         <is>
-          <t>A_TYPEFLOW_3</t>
+          <t>A_TYPEACCOUNT_0</t>
         </is>
       </c>
       <c r="B365" s="4" t="inlineStr">
         <is>
-          <t>K_TYPEFLOW</t>
+          <t>K_TYPEACCOUNT</t>
         </is>
       </c>
       <c r="C365" s="4" t="inlineStr">
         <is>
-          <t>Private Leistungen zu marktüblichen Bedingungen (Nettoausgaben)</t>
+          <t>Girokonten</t>
         </is>
       </c>
       <c r="D365" s="4" t="inlineStr">
         <is>
-          <t>Private sector flows at market terms (net disbursement)</t>
+          <t>Current accounts</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="366">
       <c r="A366" s="4" t="inlineStr">
         <is>
-          <t>A_TYPEFLOW_4</t>
+          <t>A_TYPEACCOUNT_1</t>
         </is>
       </c>
       <c r="B366" s="4" t="inlineStr">
         <is>
-          <t>K_TYPEFLOW</t>
+          <t>K_TYPEACCOUNT</t>
         </is>
       </c>
       <c r="C366" s="4" t="inlineStr">
         <is>
-          <t>Leistungen von Nichtregierungsorganisationen aus Eigenmitteln (Nettoausgaben)</t>
+          <t>Online-Konten</t>
         </is>
       </c>
       <c r="D366" s="4" t="inlineStr">
         <is>
-          <t>Private concessional flows (net disbursements)</t>
+          <t>Online accounts</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="367">
       <c r="A367" s="4" t="inlineStr">
         <is>
-          <t>A_TYPEWASTE_0</t>
+          <t>A_TYPEBIOMASS_1</t>
         </is>
       </c>
       <c r="B367" s="4" t="inlineStr">
         <is>
-          <t>K_TYPEWASTE</t>
+          <t>K_TYPEBIOMASS</t>
         </is>
       </c>
       <c r="C367" s="4" t="inlineStr">
         <is>
-          <t>Abfallaufkommen insgesamt</t>
+          <t>Stehendes Holz</t>
         </is>
       </c>
       <c r="D367" s="4" t="inlineStr">
         <is>
-          <t>Total waste</t>
+          <t>Standig wood</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="368">
       <c r="A368" s="4" t="inlineStr">
         <is>
-          <t>A_TYPEWASTE_1</t>
+          <t>A_TYPEBIOMASS_2</t>
         </is>
       </c>
       <c r="B368" s="4" t="inlineStr">
         <is>
-          <t>K_TYPEWASTE</t>
+          <t>K_TYPEBIOMASS</t>
         </is>
       </c>
       <c r="C368" s="4" t="inlineStr">
         <is>
-          <t>Siedlungsabfälle insgesamt</t>
+          <t>Sonstige Holzbiomasse</t>
         </is>
       </c>
       <c r="D368" s="4" t="inlineStr">
         <is>
-          <t>Municipal waste</t>
+          <t>Other woody biomass</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="369">
       <c r="A369" s="4" t="inlineStr">
         <is>
-          <t>A_TYPHARRAS_NONSEX</t>
+          <t>A_TYPEBIOMASS_3</t>
         </is>
       </c>
       <c r="B369" s="4" t="inlineStr">
         <is>
-          <t>K_TYPHARRAS</t>
+          <t>K_TYPEBIOMASS</t>
         </is>
       </c>
       <c r="C369" s="4" t="inlineStr">
         <is>
-          <t>Nicht-sexuelle Belästigung</t>
+          <t>Sonstige Biomasse in Wäldern</t>
         </is>
       </c>
       <c r="D369" s="4" t="inlineStr">
         <is>
-          <t>Non-sexual harassment</t>
+          <t>Other biomass in forests</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="370">
       <c r="A370" s="4" t="inlineStr">
         <is>
-          <t>A_TYPHARRAS_SEX</t>
+          <t>A_TYPECLASS_FAO</t>
         </is>
       </c>
       <c r="B370" s="4" t="inlineStr">
         <is>
-          <t>K_TYPHARRAS</t>
+          <t>K_TYPECLASS</t>
         </is>
       </c>
       <c r="C370" s="4" t="inlineStr">
         <is>
-          <t>Sexuelle Belästigung</t>
+          <t>FAO-Klassifikation</t>
         </is>
       </c>
       <c r="D370" s="4" t="inlineStr">
         <is>
-          <t>Sexual harassment</t>
+          <t>FAO classification</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="371">
       <c r="A371" s="4" t="inlineStr">
         <is>
-          <t>A_TYPIFICATION_RURAL</t>
+          <t>A_TYPECLASS_NAT</t>
         </is>
       </c>
       <c r="B371" s="4" t="inlineStr">
         <is>
-          <t>K_URBAN</t>
+          <t>K_TYPECLASS</t>
         </is>
       </c>
       <c r="C371" s="4" t="inlineStr">
         <is>
-          <t>Ländliche Gebiete</t>
+          <t>Nationale Klassifikation</t>
         </is>
       </c>
       <c r="D371" s="4" t="inlineStr">
         <is>
-          <t>Rural areas</t>
+          <t>National classification</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="372">
       <c r="A372" s="4" t="inlineStr">
         <is>
-          <t>A_TYPIFICATION_SUBURBS</t>
+          <t>A_TYPEEXPLOITATION_1</t>
         </is>
       </c>
       <c r="B372" s="4" t="inlineStr">
         <is>
-          <t>K_URBAN</t>
+          <t>K_TYPEEXPLOITATION</t>
         </is>
       </c>
       <c r="C372" s="4" t="inlineStr">
         <is>
-          <t>Kleinere Städte und Vororte</t>
+          <t>Arbeitsausbeutung</t>
         </is>
       </c>
       <c r="D372" s="4" t="inlineStr">
         <is>
-          <t>Towns and suburbs</t>
+          <t>Labour exploitation</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="373">
       <c r="A373" s="4" t="inlineStr">
         <is>
-          <t>A_TYPIFICATION_URBAN</t>
+          <t>A_TYPEEXPLOITATION_2</t>
         </is>
       </c>
       <c r="B373" s="4" t="inlineStr">
         <is>
-          <t>K_URBAN</t>
+          <t>K_TYPEEXPLOITATION</t>
         </is>
       </c>
       <c r="C373" s="4" t="inlineStr">
         <is>
-          <t>Städte</t>
+          <t>Sexuelle Ausbeutung</t>
         </is>
       </c>
       <c r="D373" s="4" t="inlineStr">
         <is>
-          <t>Cities</t>
+          <t>Sexual exploitation</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="374">
       <c r="A374" s="4" t="inlineStr">
         <is>
-          <t>A_TYPIFICATION_URBAN2</t>
+          <t>A_TYPEFLOW_0</t>
         </is>
       </c>
       <c r="B374" s="4" t="inlineStr">
         <is>
-          <t>K_URBAN</t>
+          <t>K_TYPEFLOW</t>
         </is>
       </c>
       <c r="C374" s="4" t="inlineStr">
         <is>
-          <t>Städte</t>
+          <t>Sonstige öffentliche Nettoausgaben (OOF)</t>
         </is>
       </c>
       <c r="D374" s="4" t="inlineStr">
         <is>
-          <t>Urban</t>
+          <t>OOF (net disbursements)</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="375">
       <c r="A375" s="4" t="inlineStr">
         <is>
-          <t>A_TYPPSYCHVIOL_1</t>
+          <t>A_TYPEFLOW_1</t>
         </is>
       </c>
       <c r="B375" s="4" t="inlineStr">
         <is>
-          <t>K_TYPPSYCHVIOL</t>
+          <t>K_TYPEFLOW</t>
         </is>
       </c>
       <c r="C375" s="4" t="inlineStr">
         <is>
-          <t>Persönliche Beleidigung im Internet</t>
+          <t>Öffentlich unterstützte Exportkredite (Nettoausgaben)</t>
         </is>
       </c>
       <c r="D375" s="4" t="inlineStr">
         <is>
-          <t>Personal offense on the Internet</t>
+          <t>Officially supported export credits (net disbursements)</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="376">
       <c r="A376" s="4" t="inlineStr">
         <is>
-          <t>A_TYPPSYCHVIOL_2</t>
+          <t>A_TYPEFLOW_2</t>
         </is>
       </c>
       <c r="B376" s="4" t="inlineStr">
         <is>
-          <t>K_TYPPSYCHVIOL</t>
+          <t>K_TYPEFLOW</t>
         </is>
       </c>
       <c r="C376" s="4" t="inlineStr">
         <is>
-          <t>Gewaltandrohung offline</t>
+          <t>Öffentliche Nettoentwicklungsausgaben (ODA)</t>
         </is>
       </c>
       <c r="D376" s="4" t="inlineStr">
         <is>
-          <t>Threat of violence offline</t>
+          <t>ODA (net disbursements)</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="377">
       <c r="A377" s="4" t="inlineStr">
         <is>
-          <t>A_TYPPSYCHVIOL_3</t>
+          <t>A_TYPEFLOW_3</t>
         </is>
       </c>
       <c r="B377" s="4" t="inlineStr">
         <is>
-          <t>K_TYPPSYCHVIOL</t>
+          <t>K_TYPEFLOW</t>
         </is>
       </c>
       <c r="C377" s="4" t="inlineStr">
         <is>
-          <t>Gewaltandrohung online</t>
+          <t>Private Leistungen zu marktüblichen Bedingungen (Nettoausgaben)</t>
         </is>
       </c>
       <c r="D377" s="4" t="inlineStr">
         <is>
-          <t>Threat of violence online</t>
+          <t>Private sector flows at market terms (net disbursement)</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="378">
       <c r="A378" s="4" t="inlineStr">
         <is>
-          <t>A_TYPSEXVIOL_1</t>
+          <t>A_TYPEFLOW_4</t>
         </is>
       </c>
       <c r="B378" s="4" t="inlineStr">
         <is>
-          <t>K_TYPSEXVIOL</t>
+          <t>K_TYPEFLOW</t>
         </is>
       </c>
       <c r="C378" s="4" t="inlineStr">
         <is>
-          <t>Zeigen von Geschlechtsteilen</t>
+          <t>Leistungen von Nichtregierungsorganisationen aus Eigenmitteln (Nettoausgaben)</t>
         </is>
       </c>
       <c r="D378" s="4" t="inlineStr">
         <is>
-          <t>Exposure of genitals</t>
+          <t>Private concessional flows (net disbursements)</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="379">
       <c r="A379" s="4" t="inlineStr">
         <is>
-          <t>A_TYPSEXVIOL_2</t>
+          <t>A_TYPEWASTE_0</t>
         </is>
       </c>
       <c r="B379" s="4" t="inlineStr">
         <is>
-          <t>K_TYPSEXVIOL</t>
+          <t>K_TYPEWASTE</t>
         </is>
       </c>
       <c r="C379" s="4" t="inlineStr">
         <is>
-          <t>Körperliche sexuelle Belästigung</t>
+          <t>Abfallaufkommen insgesamt</t>
         </is>
       </c>
       <c r="D379" s="4" t="inlineStr">
         <is>
-          <t>Physical sexual assault</t>
+          <t>Total waste</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="380">
       <c r="A380" s="4" t="inlineStr">
         <is>
-          <t>A_TYPSEXVIOL_3</t>
+          <t>A_TYPEWASTE_1</t>
         </is>
       </c>
       <c r="B380" s="4" t="inlineStr">
         <is>
-          <t>K_TYPSEXVIOL</t>
+          <t>K_TYPEWASTE</t>
         </is>
       </c>
       <c r="C380" s="4" t="inlineStr">
         <is>
-          <t>Sexueller Missbrauch oder Vergewaltigung</t>
+          <t>Siedlungsabfälle insgesamt</t>
         </is>
       </c>
       <c r="D380" s="4" t="inlineStr">
         <is>
-          <t>Sexual abuse or rape</t>
+          <t>Municipal waste</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="381">
       <c r="A381" s="4" t="inlineStr">
         <is>
-          <t>A_TYPVIOL_A_PHYS</t>
+          <t>A_TYPHARRAS_NONSEX</t>
         </is>
       </c>
       <c r="B381" s="4" t="inlineStr">
         <is>
-          <t>K_TYPVIOL</t>
+          <t>K_TYPHARRAS</t>
         </is>
       </c>
       <c r="C381" s="4" t="inlineStr">
         <is>
-          <t>a) Physische Gewalt</t>
+          <t>Nicht-sexuelle Belästigung</t>
         </is>
       </c>
       <c r="D381" s="4" t="inlineStr">
         <is>
-          <t>a) Physical violence</t>
+          <t>Non-sexual harassment</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="382">
       <c r="A382" s="4" t="inlineStr">
         <is>
-          <t>A_TYPVIOL_ASSAULT</t>
+          <t>A_TYPHARRAS_SEX</t>
         </is>
       </c>
       <c r="B382" s="4" t="inlineStr">
         <is>
-          <t>K_TYPPHYSVIOL</t>
+          <t>K_TYPHARRAS</t>
         </is>
       </c>
       <c r="C382" s="4" t="inlineStr">
         <is>
-          <t>Körperverletzung</t>
+          <t>Sexuelle Belästigung</t>
         </is>
       </c>
       <c r="D382" s="4" t="inlineStr">
         <is>
-          <t>Physical assault</t>
+          <t>Sexual harassment</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="383">
       <c r="A383" s="4" t="inlineStr">
         <is>
-          <t>A_TYPVIOL_B_PSYCH</t>
+          <t>A_TYPIFICATION_RURAL</t>
         </is>
       </c>
       <c r="B383" s="4" t="inlineStr">
         <is>
-          <t>K_TYPVIOL</t>
+          <t>K_URBAN</t>
         </is>
       </c>
       <c r="C383" s="4" t="inlineStr">
         <is>
-          <t>b) Psychische Gewalt</t>
+          <t>Ländliche Gebiete</t>
         </is>
       </c>
       <c r="D383" s="4" t="inlineStr">
         <is>
-          <t>b) Psychological violence</t>
+          <t>Rural areas</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="384">
       <c r="A384" s="4" t="inlineStr">
         <is>
-          <t>A_TYPVIOL_C_SEX</t>
+          <t>A_TYPIFICATION_SUBURBS</t>
         </is>
       </c>
       <c r="B384" s="4" t="inlineStr">
         <is>
-          <t>K_TYPVIOL</t>
+          <t>K_URBAN</t>
         </is>
       </c>
       <c r="C384" s="4" t="inlineStr">
         <is>
-          <t>c) Sexuelle Gewalt</t>
+          <t>Kleinere Städte und Vororte</t>
         </is>
       </c>
       <c r="D384" s="4" t="inlineStr">
         <is>
-          <t>c) Sexual violence</t>
+          <t>Towns and suburbs</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="385">
       <c r="A385" s="4" t="inlineStr">
         <is>
-          <t>A_TYPVIOL_ROBBERY</t>
+          <t>A_TYPIFICATION_URBAN</t>
         </is>
       </c>
       <c r="B385" s="4" t="inlineStr">
         <is>
-          <t>K_TYPPHYSVIOL</t>
+          <t>K_URBAN</t>
         </is>
       </c>
       <c r="C385" s="4" t="inlineStr">
         <is>
-          <t>Raub</t>
+          <t>Städte</t>
         </is>
       </c>
       <c r="D385" s="4" t="inlineStr">
         <is>
-          <t>Robbery</t>
+          <t>Cities</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="386">
       <c r="A386" s="4" t="inlineStr">
         <is>
-          <t>A_UNPAID_CARE</t>
+          <t>A_TYPIFICATION_URBAN2</t>
         </is>
       </c>
       <c r="B386" s="4" t="inlineStr">
         <is>
-          <t>K_UNPAIDWORK</t>
+          <t>K_URBAN</t>
         </is>
       </c>
       <c r="C386" s="4" t="inlineStr">
         <is>
-          <t>Pflegearbeit</t>
+          <t>Städte</t>
         </is>
       </c>
       <c r="D386" s="4" t="inlineStr">
         <is>
-          <t>Care work</t>
+          <t>Urban</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="387">
       <c r="A387" s="4" t="inlineStr">
         <is>
-          <t>A_UNPAID_HOUSE</t>
+          <t>A_TYPPSYCHVIOL_1</t>
         </is>
       </c>
       <c r="B387" s="4" t="inlineStr">
         <is>
-          <t>K_UNPAIDWORK</t>
+          <t>K_TYPPSYCHVIOL</t>
         </is>
       </c>
       <c r="C387" s="4" t="inlineStr">
         <is>
-          <t>Hausarbeit</t>
+          <t>Persönliche Beleidigung im Internet</t>
         </is>
       </c>
       <c r="D387" s="4" t="inlineStr">
         <is>
-          <t>Domestic work</t>
+          <t>Personal offense on the Internet</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="388">
       <c r="A388" s="4" t="inlineStr">
         <is>
-          <t>A_UNPAID_HOUSE_CARE</t>
+          <t>A_TYPPSYCHVIOL_2</t>
         </is>
       </c>
       <c r="B388" s="4" t="inlineStr">
         <is>
-          <t>K_UNPAIDWORK</t>
+          <t>K_TYPPSYCHVIOL</t>
         </is>
       </c>
       <c r="C388" s="4" t="inlineStr">
         <is>
-          <t>Haus- und Pflegearbeit</t>
+          <t>Gewaltandrohung offline</t>
         </is>
       </c>
       <c r="D388" s="4" t="inlineStr">
         <is>
-          <t>Domestic and care work</t>
+          <t>Threat of violence offline</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="389">
       <c r="A389" s="4" t="inlineStr">
         <is>
-          <t>A_VERW_ZWECK</t>
+          <t>A_TYPPSYCHVIOL_3</t>
         </is>
       </c>
       <c r="B389" s="4" t="inlineStr">
         <is>
-          <t>K_SERIES</t>
+          <t>K_TYPPSYCHVIOL</t>
         </is>
       </c>
       <c r="C389" s="4" t="inlineStr">
         <is>
-          <t>Verwandte Zwecke</t>
+          <t>Gewaltandrohung online</t>
         </is>
       </c>
       <c r="D389" s="4" t="inlineStr">
         <is>
-          <t>Other related purposes</t>
+          <t>Threat of violence online</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="390">
       <c r="A390" s="4" t="inlineStr">
         <is>
-          <t>A_WASTETREATMNT_0</t>
+          <t>A_TYPSEXVIOL_1</t>
         </is>
       </c>
       <c r="B390" s="4" t="inlineStr">
         <is>
-          <t>K_WASTETREATMNT</t>
+          <t>K_TYPSEXVIOL</t>
         </is>
       </c>
       <c r="C390" s="4" t="inlineStr">
         <is>
-          <t>Ablagerung auf oder im Boden und Bodenbehandlung und Freisetzung in Gewässern</t>
+          <t>Zeigen von Geschlechtsteilen</t>
         </is>
       </c>
       <c r="D390" s="4" t="inlineStr">
         <is>
-          <t>Deposit onto or into land and land treatment and release into water bodies</t>
+          <t>Exposure of genitals</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="391">
       <c r="A391" s="4" t="inlineStr">
         <is>
-          <t>A_WASTETREATMNT_1</t>
+          <t>A_TYPSEXVIOL_2</t>
         </is>
       </c>
       <c r="B391" s="4" t="inlineStr">
         <is>
-          <t>K_WASTETREATMNT</t>
+          <t>K_TYPSEXVIOL</t>
         </is>
       </c>
       <c r="C391" s="4" t="inlineStr">
         <is>
-          <t>Energierückgewinnung</t>
+          <t>Körperliche sexuelle Belästigung</t>
         </is>
       </c>
       <c r="D391" s="4" t="inlineStr">
         <is>
-          <t>Energy recovery</t>
+          <t>Physical sexual assault</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="392">
       <c r="A392" s="4" t="inlineStr">
         <is>
-          <t>A_WASTETREATMNT_2</t>
+          <t>A_TYPSEXVIOL_3</t>
         </is>
       </c>
       <c r="B392" s="4" t="inlineStr">
         <is>
-          <t>K_WASTETREATMNT</t>
+          <t>K_TYPSEXVIOL</t>
         </is>
       </c>
       <c r="C392" s="4" t="inlineStr">
         <is>
-          <t>Verbrennung</t>
+          <t>Sexueller Missbrauch oder Vergewaltigung</t>
         </is>
       </c>
       <c r="D392" s="4" t="inlineStr">
         <is>
-          <t>Incineration</t>
+          <t>Sexual abuse or rape</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="393">
       <c r="A393" s="4" t="inlineStr">
         <is>
-          <t>A_WASTETREATMNT_3</t>
+          <t>A_TYPVIOL_A_PHYS</t>
         </is>
       </c>
       <c r="B393" s="4" t="inlineStr">
         <is>
-          <t>K_WASTETREATMNT</t>
+          <t>K_TYPVIOL</t>
         </is>
       </c>
       <c r="C393" s="4" t="inlineStr">
         <is>
-          <t>Verwertung anderer als die der Energierückgewinnung</t>
+          <t>a) Physische Gewalt</t>
         </is>
       </c>
       <c r="D393" s="4" t="inlineStr">
         <is>
-          <t>Recovery other than energy recovery</t>
+          <t>a) Physical violence</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="394">
       <c r="A394" s="4" t="inlineStr">
         <is>
-          <t>A_WASTEWATER_1</t>
+          <t>A_TYPVIOL_ASSAULT</t>
         </is>
       </c>
       <c r="B394" s="4" t="inlineStr">
         <is>
-          <t>K_WASTEWATER</t>
+          <t>K_TYPPHYSVIOL</t>
         </is>
       </c>
       <c r="C394" s="4" t="inlineStr">
         <is>
-          <t>Kühlwasser</t>
+          <t>Körperverletzung</t>
         </is>
       </c>
       <c r="D394" s="4" t="inlineStr">
         <is>
-          <t>Cooling water</t>
+          <t>Physical assault</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="395">
       <c r="A395" s="4" t="inlineStr">
         <is>
-          <t>A_WASTEWATER_2</t>
+          <t>A_TYPVIOL_B_PSYCH</t>
         </is>
       </c>
       <c r="B395" s="4" t="inlineStr">
         <is>
-          <t>K_WASTEWATER</t>
+          <t>K_TYPVIOL</t>
         </is>
       </c>
       <c r="C395" s="4" t="inlineStr">
         <is>
-          <t>Gesamtes produziertes Abwasser aus öffentlicher und nichtöffentlicher Entsorgung</t>
+          <t>b) Psychische Gewalt</t>
         </is>
       </c>
       <c r="D395" s="4" t="inlineStr">
         <is>
-          <t>Total wastewater produced from public and non-public disposal</t>
+          <t>b) Psychological violence</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="396">
       <c r="A396" s="4" t="inlineStr">
         <is>
-          <t>A_WATERTREATMNT_1</t>
+          <t>A_TYPVIOL_C_SEX</t>
         </is>
       </c>
       <c r="B396" s="4" t="inlineStr">
         <is>
-          <t>K_WATERTREATMNT</t>
+          <t>K_TYPVIOL</t>
         </is>
       </c>
       <c r="C396" s="4" t="inlineStr">
         <is>
-          <t>Behandeltes Abwasser</t>
+          <t>c) Sexuelle Gewalt</t>
         </is>
       </c>
       <c r="D396" s="4" t="inlineStr">
         <is>
-          <t>Treated wastewater</t>
+          <t>c) Sexual violence</t>
         </is>
       </c>
     </row>
     <row outlineLevel="0" r="397">
       <c r="A397" s="4" t="inlineStr">
         <is>
+          <t>A_TYPVIOL_ROBBERY</t>
+        </is>
+      </c>
+      <c r="B397" s="4" t="inlineStr">
+        <is>
+          <t>K_TYPPHYSVIOL</t>
+        </is>
+      </c>
+      <c r="C397" s="4" t="inlineStr">
+        <is>
+          <t>Raub</t>
+        </is>
+      </c>
+      <c r="D397" s="4" t="inlineStr">
+        <is>
+          <t>Robbery</t>
+        </is>
+      </c>
+    </row>
+    <row outlineLevel="0" r="398">
+      <c r="A398" s="4" t="inlineStr">
+        <is>
+          <t>A_UNPAID_CARE</t>
+        </is>
+      </c>
+      <c r="B398" s="4" t="inlineStr">
+        <is>
+          <t>K_UNPAIDWORK</t>
+        </is>
+      </c>
+      <c r="C398" s="4" t="inlineStr">
+        <is>
+          <t>Pflegearbeit</t>
+        </is>
+      </c>
+      <c r="D398" s="4" t="inlineStr">
+        <is>
+          <t>Care work</t>
+        </is>
+      </c>
+    </row>
+    <row outlineLevel="0" r="399">
+      <c r="A399" s="4" t="inlineStr">
+        <is>
+          <t>A_UNPAID_HOUSE</t>
+        </is>
+      </c>
+      <c r="B399" s="4" t="inlineStr">
+        <is>
+          <t>K_UNPAIDWORK</t>
+        </is>
+      </c>
+      <c r="C399" s="4" t="inlineStr">
+        <is>
+          <t>Hausarbeit</t>
+        </is>
+      </c>
+      <c r="D399" s="4" t="inlineStr">
+        <is>
+          <t>Domestic work</t>
+        </is>
+      </c>
+    </row>
+    <row outlineLevel="0" r="400">
+      <c r="A400" s="4" t="inlineStr">
+        <is>
+          <t>A_UNPAID_HOUSE_CARE</t>
+        </is>
+      </c>
+      <c r="B400" s="4" t="inlineStr">
+        <is>
+          <t>K_UNPAIDWORK</t>
+        </is>
+      </c>
+      <c r="C400" s="4" t="inlineStr">
+        <is>
+          <t>Haus- und Pflegearbeit</t>
+        </is>
+      </c>
+      <c r="D400" s="4" t="inlineStr">
+        <is>
+          <t>Domestic and care work</t>
+        </is>
+      </c>
+    </row>
+    <row outlineLevel="0" r="401">
+      <c r="A401" s="4" t="inlineStr">
+        <is>
+          <t>A_VERW_ZWECK</t>
+        </is>
+      </c>
+      <c r="B401" s="4" t="inlineStr">
+        <is>
+          <t>K_SERIES</t>
+        </is>
+      </c>
+      <c r="C401" s="4" t="inlineStr">
+        <is>
+          <t>Verwandte Zwecke</t>
+        </is>
+      </c>
+      <c r="D401" s="4" t="inlineStr">
+        <is>
+          <t>Other related purposes</t>
+        </is>
+      </c>
+    </row>
+    <row outlineLevel="0" r="402">
+      <c r="A402" s="4" t="inlineStr">
+        <is>
+          <t>A_WASTETREATMNT_0</t>
+        </is>
+      </c>
+      <c r="B402" s="4" t="inlineStr">
+        <is>
+          <t>K_WASTETREATMNT</t>
+        </is>
+      </c>
+      <c r="C402" s="4" t="inlineStr">
+        <is>
+          <t>Ablagerung auf oder im Boden und Bodenbehandlung und Freisetzung in Gewässern</t>
+        </is>
+      </c>
+      <c r="D402" s="4" t="inlineStr">
+        <is>
+          <t>Deposit onto or into land and land treatment and release into water bodies</t>
+        </is>
+      </c>
+    </row>
+    <row outlineLevel="0" r="403">
+      <c r="A403" s="4" t="inlineStr">
+        <is>
+          <t>A_WASTETREATMNT_1</t>
+        </is>
+      </c>
+      <c r="B403" s="4" t="inlineStr">
+        <is>
+          <t>K_WASTETREATMNT</t>
+        </is>
+      </c>
+      <c r="C403" s="4" t="inlineStr">
+        <is>
+          <t>Energierückgewinnung</t>
+        </is>
+      </c>
+      <c r="D403" s="4" t="inlineStr">
+        <is>
+          <t>Energy recovery</t>
+        </is>
+      </c>
+    </row>
+    <row outlineLevel="0" r="404">
+      <c r="A404" s="4" t="inlineStr">
+        <is>
+          <t>A_WASTETREATMNT_2</t>
+        </is>
+      </c>
+      <c r="B404" s="4" t="inlineStr">
+        <is>
+          <t>K_WASTETREATMNT</t>
+        </is>
+      </c>
+      <c r="C404" s="4" t="inlineStr">
+        <is>
+          <t>Verbrennung</t>
+        </is>
+      </c>
+      <c r="D404" s="4" t="inlineStr">
+        <is>
+          <t>Incineration</t>
+        </is>
+      </c>
+    </row>
+    <row outlineLevel="0" r="405">
+      <c r="A405" s="4" t="inlineStr">
+        <is>
+          <t>A_WASTETREATMNT_3</t>
+        </is>
+      </c>
+      <c r="B405" s="4" t="inlineStr">
+        <is>
+          <t>K_WASTETREATMNT</t>
+        </is>
+      </c>
+      <c r="C405" s="4" t="inlineStr">
+        <is>
+          <t>Verwertung anderer als die der Energierückgewinnung</t>
+        </is>
+      </c>
+      <c r="D405" s="4" t="inlineStr">
+        <is>
+          <t>Recovery other than energy recovery</t>
+        </is>
+      </c>
+    </row>
+    <row outlineLevel="0" r="406">
+      <c r="A406" s="4" t="inlineStr">
+        <is>
+          <t>A_WASTEWATER_1</t>
+        </is>
+      </c>
+      <c r="B406" s="4" t="inlineStr">
+        <is>
+          <t>K_WASTEWATER</t>
+        </is>
+      </c>
+      <c r="C406" s="4" t="inlineStr">
+        <is>
+          <t>Kühlwasser</t>
+        </is>
+      </c>
+      <c r="D406" s="4" t="inlineStr">
+        <is>
+          <t>Cooling water</t>
+        </is>
+      </c>
+    </row>
+    <row outlineLevel="0" r="407">
+      <c r="A407" s="4" t="inlineStr">
+        <is>
+          <t>A_WASTEWATER_2</t>
+        </is>
+      </c>
+      <c r="B407" s="4" t="inlineStr">
+        <is>
+          <t>K_WASTEWATER</t>
+        </is>
+      </c>
+      <c r="C407" s="4" t="inlineStr">
+        <is>
+          <t>Gesamtes produziertes Abwasser aus öffentlicher und nichtöffentlicher Entsorgung</t>
+        </is>
+      </c>
+      <c r="D407" s="4" t="inlineStr">
+        <is>
+          <t>Total wastewater produced from public and non-public disposal</t>
+        </is>
+      </c>
+    </row>
+    <row outlineLevel="0" r="408">
+      <c r="A408" s="4" t="inlineStr">
+        <is>
+          <t>A_WATERTREATMNT_1</t>
+        </is>
+      </c>
+      <c r="B408" s="4" t="inlineStr">
+        <is>
+          <t>K_WATERTREATMNT</t>
+        </is>
+      </c>
+      <c r="C408" s="4" t="inlineStr">
+        <is>
+          <t>Behandeltes Abwasser</t>
+        </is>
+      </c>
+      <c r="D408" s="4" t="inlineStr">
+        <is>
+          <t>Treated wastewater</t>
+        </is>
+      </c>
+    </row>
+    <row outlineLevel="0" r="409">
+      <c r="A409" s="4" t="inlineStr">
+        <is>
           <t>A_WATERTREATMNT_2</t>
         </is>
       </c>
-      <c r="B397" s="4" t="inlineStr">
+      <c r="B409" s="4" t="inlineStr">
         <is>
           <t>K_WATERTREATMNT</t>
         </is>
       </c>
-      <c r="C397" s="4" t="inlineStr">
+      <c r="C409" s="4" t="inlineStr">
         <is>
           <t>Unbehandeltes Abwasser</t>
         </is>
       </c>
-      <c r="D397" s="4" t="inlineStr">
+      <c r="D409" s="4" t="inlineStr">
         <is>
           <t>Untreated wastewater</t>
         </is>

</xml_diff>